<commit_message>
Kalkulator NK38: rozładunek jednorazowo, konserwacja A/B, oferta z adresatem w polach
- rozładunek sprzętu to jedna kwota (przyjazd i wyjazd wózka), nie mnożona przez TIR
- konserwacja A/B w zł/MP/mies., w nagłówku cena roczna i półroczna
- oferta: data dzisiejsza, numer RRRRMMDDGG/INK (+A, B… w tej samej godzinie),
  nazwa pliku jak w ofertach, adresat w osobnych polach, H1/H2/długość/prześwit
  w danych inwestycji, wysokości pojazdów liczone automatycznie, Pozycja 1 / Opcja 1,
  czas montażu do ręcznej zmiany, Verdana 8 pt, logo firmowe domyślnie
- przycisk Oferta Word na górnym pasku

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/Kalkulator_NK38_v1.xlsx
+++ b/kalkulator-nk38/Kalkulator_NK38_v1.xlsx
@@ -33,9 +33,6 @@
     <definedName function="false" hidden="false" name="c_km_dzien" vbProcedure="false">Cennik!$C$53</definedName>
     <definedName function="false" hidden="false" name="c_km_krakow" vbProcedure="false">Cennik!$C$52</definedName>
     <definedName function="false" hidden="false" name="c_kob" vbProcedure="false">Cennik!$C$65</definedName>
-    <definedName function="false" hidden="false" name="c_konserw" vbProcedure="false">Cennik!$C$69</definedName>
-    <definedName function="false" hidden="false" name="c_konserw2" vbProcedure="false">Cennik!$C$70</definedName>
-    <definedName function="false" hidden="false" name="c_konserw3" vbProcedure="false">Cennik!$C$71</definedName>
     <definedName function="false" hidden="false" name="c_magistrala" vbProcedure="false">Cennik!$C$26</definedName>
     <definedName function="false" hidden="false" name="c_mal_bar" vbProcedure="false">Cennik!$C$35</definedName>
     <definedName function="false" hidden="false" name="c_mal_D" vbProcedure="false">Cennik!$C$34</definedName>
@@ -80,7 +77,7 @@
     <definedName function="false" hidden="false" name="e_podr_pom" vbProcedure="false">Obliczenia!$C$32</definedName>
     <definedName function="false" hidden="false" name="e_rozl_dni" vbProcedure="false">Obliczenia!$C$31</definedName>
     <definedName function="false" hidden="false" name="in_agregaty" vbProcedure="false">Dane!$C$22</definedName>
-    <definedName function="false" hidden="false" name="in_analiza" vbProcedure="false">Dane!$C$60</definedName>
+    <definedName function="false" hidden="false" name="in_analiza" vbProcedure="false">Dane!$C$62</definedName>
     <definedName function="false" hidden="false" name="in_barierki" vbProcedure="false">Dane!$C$24</definedName>
     <definedName function="false" hidden="false" name="in_D" vbProcedure="false">Dane!$C$20</definedName>
     <definedName function="false" hidden="false" name="in_data" vbProcedure="false">Dane!$C$7</definedName>
@@ -96,6 +93,8 @@
     <definedName function="false" hidden="false" name="in_km" vbProcedure="false">Dane!$C$13</definedName>
     <definedName function="false" hidden="false" name="in_km_mon" vbProcedure="false">Dane!$C$15</definedName>
     <definedName function="false" hidden="false" name="in_km_pom" vbProcedure="false">Dane!$C$14</definedName>
+    <definedName function="false" hidden="false" name="in_konsA" vbProcedure="false">Dane!$C$60</definedName>
+    <definedName function="false" hidden="false" name="in_konsB" vbProcedure="false">Dane!$C$61</definedName>
     <definedName function="false" hidden="false" name="in_lok" vbProcedure="false">Dane!$C$12</definedName>
     <definedName function="false" hidden="false" name="in_magistrala" vbProcedure="false">Dane!$C$23</definedName>
     <definedName function="false" hidden="false" name="in_maskownice" vbProcedure="false">Dane!$C$25</definedName>
@@ -141,12 +140,12 @@
     <definedName function="false" hidden="false" name="m_suma_2500" vbProcedure="false">Obliczenia!$C$22</definedName>
     <definedName function="false" hidden="false" name="m_utr" vbProcedure="false">Obliczenia!$C$25</definedName>
     <definedName function="false" hidden="false" name="m_utr_auto" vbProcedure="false">Obliczenia!$C$24</definedName>
-    <definedName function="false" hidden="false" name="t_gl_doplata" vbProcedure="false">Cennik!$C$75:$C$83</definedName>
-    <definedName function="false" hidden="false" name="t_gl_silownik" vbProcedure="false">Cennik!$D$75:$D$83</definedName>
-    <definedName function="false" hidden="false" name="t_sk_cena" vbProcedure="false">Cennik!$C$87:$C$113</definedName>
-    <definedName function="false" hidden="false" name="t_sk_D" vbProcedure="false">Cennik!$E$87:$E$113</definedName>
-    <definedName function="false" hidden="false" name="t_sk_grupa" vbProcedure="false">Cennik!$F$87:$F$113</definedName>
-    <definedName function="false" hidden="false" name="t_sk_S" vbProcedure="false">Cennik!$D$87:$D$113</definedName>
+    <definedName function="false" hidden="false" name="t_gl_doplata" vbProcedure="false">Cennik!$C$71:$C$79</definedName>
+    <definedName function="false" hidden="false" name="t_gl_silownik" vbProcedure="false">Cennik!$D$71:$D$79</definedName>
+    <definedName function="false" hidden="false" name="t_sk_cena" vbProcedure="false">Cennik!$C$83:$C$109</definedName>
+    <definedName function="false" hidden="false" name="t_sk_D" vbProcedure="false">Cennik!$E$83:$E$109</definedName>
+    <definedName function="false" hidden="false" name="t_sk_grupa" vbProcedure="false">Cennik!$F$83:$F$109</definedName>
+    <definedName function="false" hidden="false" name="t_sk_S" vbProcedure="false">Cennik!$D$83:$D$109</definedName>
     <definedName function="false" hidden="false" name="t_wymiary" vbProcedure="false">Dane!$F$46</definedName>
     <definedName function="false" hidden="false" name="t_zaglebienia" vbProcedure="false">Dane!$F$45</definedName>
   </definedNames>
@@ -160,7 +159,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="358">
   <si>
     <t xml:space="preserve">KALKULATOR NK38 - DANE WEJŚCIOWE</t>
   </si>
@@ -327,10 +326,10 @@
     <t xml:space="preserve">Orientacyjnie: KRK 1600, WAW/WRO 3300, POZ/ZG 4500</t>
   </si>
   <si>
-    <t xml:space="preserve">Rozładunek - sprzęt / TIR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WAW 1700, KRK 500</t>
+    <t xml:space="preserve">Rozładunek - sprzęt (jednorazowo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jednorazowy koszt przyjazdu i wyjazdu wózka</t>
   </si>
   <si>
     <t xml:space="preserve">Nadpisz: dni rozładunku</t>
@@ -375,6 +374,12 @@
     <t xml:space="preserve">Kurs EUR/PLN</t>
   </si>
   <si>
+    <t xml:space="preserve">Konserwacja - cena A [zł / MP / miesiąc]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Konserwacja - cena B [zł / MP / miesiąc]</t>
+  </si>
+  <si>
     <t xml:space="preserve">Analiza liczby osób dla wariantu</t>
   </si>
   <si>
@@ -540,7 +545,7 @@
     <t xml:space="preserve">Dopłata Q=2500</t>
   </si>
   <si>
-    <t xml:space="preserve">Konserwacja roczna (40 / 45 / 50 zł/MP/mies.)</t>
+    <t xml:space="preserve">Konserwacja roczna A / B</t>
   </si>
   <si>
     <t xml:space="preserve">Opis / wariant</t>
@@ -564,6 +569,9 @@
     <t xml:space="preserve">• Czas podróży: wzór 'Stary (poprawiony)' = stary dla &lt; 800 km, dla &gt;= 800 km uwzględnia liczbę wyjazdów. 'Uproszczony' = 2 x km / 650 km dziennie na wyjazd.</t>
   </si>
   <si>
+    <t xml:space="preserve">• Rozładunek sprzętu to jednorazowy koszt przyjazdu i wyjazdu wózka (nie mnoży się przez liczbę TIR-ów).</t>
+  </si>
+  <si>
     <t xml:space="preserve">• Zysk B liczony od tych samych kosztów co zysk A (dawna kolumna N, bez zmiany ceny dźwigu).</t>
   </si>
   <si>
@@ -909,27 +917,6 @@
     <t xml:space="preserve">KAL!J37</t>
   </si>
   <si>
-    <t xml:space="preserve">Serwis (informacyjnie)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Konserwacja zł / MP / miesiąc (wariant 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KAL!I45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Konserwacja zł / MP / miesiąc (wariant 2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KAL!L45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Konserwacja zł / MP / miesiąc (wariant 3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KAL!N45</t>
-  </si>
-  <si>
     <t xml:space="preserve">Zagłębienia (standard 170 cm: bez dopłaty, siłownik 1700)</t>
   </si>
   <si>
@@ -1197,7 +1184,7 @@
     <t xml:space="preserve">Spider Crane</t>
   </si>
   <si>
-    <t xml:space="preserve">Rozładunek (sprzęt)</t>
+    <t xml:space="preserve">Rozładunek (sprzęt, jednorazowo)</t>
   </si>
   <si>
     <t xml:space="preserve">Rozładunek (ludzie)</t>
@@ -1835,7 +1822,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:F68"/>
+  <dimension ref="B2:F70"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2410,39 +2397,37 @@
       <c r="B60" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="C60" s="6" t="s">
+      <c r="C60" s="13" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B61" s="0" t="s">
         <v>72</v>
       </c>
+      <c r="C61" s="13" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B62" s="4" t="s">
+      <c r="B62" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="C62" s="5"/>
-      <c r="D62" s="5"/>
-      <c r="E62" s="5"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="16" t="str">
-        <f aca="false">IF(OR(C39&lt;0,D39&lt;0),"BŁĄD: więcej zagłębień niż platform","ok")</f>
-        <v>ok</v>
-      </c>
-      <c r="C63" s="16"/>
-      <c r="D63" s="16"/>
-      <c r="E63" s="16"/>
+      <c r="C62" s="6" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="16" t="str">
-        <f aca="false">IF(OR(in_szer1_S+in_szer2_S&gt;in_S,in_szer1_D+in_szer2_D&gt;in_D),"BŁĄD: więcej szerokości niż platform","ok")</f>
-        <v>ok</v>
-      </c>
-      <c r="C64" s="16"/>
-      <c r="D64" s="16"/>
-      <c r="E64" s="16"/>
+      <c r="B64" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C64" s="5"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="16" t="str">
-        <f aca="false">IF(OR(in_dl500_S+in_dl540_S+in_dl550_S&gt;in_S,in_dl500_D+in_dl540_D+in_dl550_D&gt;in_D),"BŁĄD: więcej długości niż platform","ok")</f>
+        <f aca="false">IF(OR(C39&lt;0,D39&lt;0),"BŁĄD: więcej zagłębień niż platform","ok")</f>
         <v>ok</v>
       </c>
       <c r="C65" s="16"/>
@@ -2451,7 +2436,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="16" t="str">
-        <f aca="false">IF(in_agregaty*6&lt;in_S+in_D+in_NP,"UWAGA: mniej niż 1 agregat na 6 platform","ok")</f>
+        <f aca="false">IF(OR(in_szer1_S+in_szer2_S&gt;in_S,in_szer1_D+in_szer2_D&gt;in_D),"BŁĄD: więcej szerokości niż platform","ok")</f>
         <v>ok</v>
       </c>
       <c r="C66" s="16"/>
@@ -2460,8 +2445,8 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="16" t="str">
-        <f aca="false">IF(in_S+in_D+in_NP=0,"UWAGA: brak platform",IF(in_tir=0,"UWAGA: brak transportów","ok"))</f>
-        <v>UWAGA: brak platform</v>
+        <f aca="false">IF(OR(in_dl500_S+in_dl540_S+in_dl550_S&gt;in_S,in_dl500_D+in_dl540_D+in_dl550_D&gt;in_D),"BŁĄD: więcej długości niż platform","ok")</f>
+        <v>ok</v>
       </c>
       <c r="C67" s="16"/>
       <c r="D67" s="16"/>
@@ -2469,25 +2454,43 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="16" t="str">
-        <f aca="false">IF(AND(in_lok="Poza Krakowem",in_km=0),"UWAGA: brak odległości od Krakowa","ok")</f>
-        <v>UWAGA: brak odległości od Krakowa</v>
+        <f aca="false">IF(in_agregaty*6&lt;in_S+in_D+in_NP,"UWAGA: mniej niż 1 agregat na 6 platform","ok")</f>
+        <v>ok</v>
       </c>
       <c r="C68" s="16"/>
       <c r="D68" s="16"/>
       <c r="E68" s="16"/>
     </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B69" s="16" t="str">
+        <f aca="false">IF(in_S+in_D+in_NP=0,"UWAGA: brak platform",IF(in_tir=0,"UWAGA: brak transportów","ok"))</f>
+        <v>UWAGA: brak platform</v>
+      </c>
+      <c r="C69" s="16"/>
+      <c r="D69" s="16"/>
+      <c r="E69" s="16"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B70" s="16" t="str">
+        <f aca="false">IF(AND(in_lok="Poza Krakowem",in_km=0),"UWAGA: brak odległości od Krakowa","ok")</f>
+        <v>UWAGA: brak odległości od Krakowa</v>
+      </c>
+      <c r="C70" s="16"/>
+      <c r="D70" s="16"/>
+      <c r="E70" s="16"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="B64:E64"/>
     <mergeCell ref="B65:E65"/>
     <mergeCell ref="B66:E66"/>
     <mergeCell ref="B67:E67"/>
     <mergeCell ref="B68:E68"/>
+    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="B70:E70"/>
   </mergeCells>
-  <conditionalFormatting sqref="B63:B68">
+  <conditionalFormatting sqref="B65:B70">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>B63&lt;&gt;"ok"</formula>
+      <formula>B65&lt;&gt;"ok"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
@@ -2503,7 +2506,7 @@
       <formula1>"Stary (poprawiony),Uproszczony"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C60" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C62" type="list">
       <formula1>"2000 kg,2500 kg,2000 kg + słupki,2500 kg + słupki"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2531,7 +2534,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:H68"/>
+  <dimension ref="B2:H69"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2542,7 +2545,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2565,19 +2568,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2626,7 +2629,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C9" s="19" t="n">
         <f aca="false">Obliczenia!D73</f>
@@ -2647,7 +2650,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C10" s="19" t="n">
         <f aca="false">Obliczenia!D78</f>
@@ -2668,7 +2671,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C11" s="20" t="n">
         <f aca="false">Obliczenia!D74</f>
@@ -2689,7 +2692,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C12" s="19" t="n">
         <f aca="false">Obliczenia!D69</f>
@@ -2710,7 +2713,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C13" s="19" t="n">
         <f aca="false">Obliczenia!D76</f>
@@ -2731,7 +2734,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="0" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C14" s="19" t="n">
         <f aca="false">Obliczenia!D72</f>
@@ -2752,7 +2755,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C16" s="19" t="n">
         <f aca="false">Obliczenia!D54</f>
@@ -2773,7 +2776,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="0" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C17" s="19" t="n">
         <f aca="false">Obliczenia!D55</f>
@@ -2794,7 +2797,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="0" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C18" s="19" t="n">
         <f aca="false">Obliczenia!D58+Obliczenia!D59+Obliczenia!D60</f>
@@ -2815,7 +2818,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="0" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C19" s="19" t="n">
         <f aca="false">Obliczenia!D63+Obliczenia!D61+Obliczenia!D62</f>
@@ -2836,7 +2839,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="0" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C20" s="19" t="n">
         <f aca="false">Obliczenia!D57+Obliczenia!D64+Obliczenia!D56</f>
@@ -2857,7 +2860,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="0" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C21" s="19" t="n">
         <f aca="false">Obliczenia!D67+Obliczenia!D68+Obliczenia!D70</f>
@@ -2878,7 +2881,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C23" s="21" t="n">
         <f aca="false">Obliczenia!D51</f>
@@ -2899,7 +2902,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="11" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C24" s="21" t="n">
         <f aca="false">Obliczenia!D52</f>
@@ -2920,7 +2923,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="0" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C25" s="22" t="n">
         <f aca="false">Obliczenia!D50</f>
@@ -2941,18 +2944,18 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="0" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C28" s="19" t="n">
         <f aca="false">Obliczenia!F71-Obliczenia!D71</f>
@@ -2965,7 +2968,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="0" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C29" s="19" t="n">
         <f aca="false">Obliczenia!F71-Obliczenia!D71+(c_slupek22-c_slupek)*m_MP*e_mnoznik</f>
@@ -2978,7 +2981,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="0" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C30" s="19" t="n">
         <f aca="false">m_malowanie*e_mnoznik</f>
@@ -2997,30 +3000,30 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F33" s="17" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G33" s="17" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H33" s="17" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C34" s="19" t="n">
         <f aca="false">Obliczenia!I71</f>
@@ -3049,7 +3052,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C35" s="19" t="n">
         <f aca="false">Obliczenia!I73</f>
@@ -3078,7 +3081,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="0" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C36" s="23" t="n">
         <f aca="false">Obliczenia!I51</f>
@@ -3107,7 +3110,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C37" s="23" t="n">
         <f aca="false">Obliczenia!I48</f>
@@ -3136,7 +3139,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C38" s="19" t="n">
         <f aca="false">Obliczenia!I57+Obliczenia!I64</f>
@@ -3165,12 +3168,12 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
@@ -3179,7 +3182,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C42" s="16" t="str">
         <f aca="false">in_typ&amp;": "&amp;IF(in_S&gt;0,in_S&amp;" x S (2 MP)  ","")&amp;IF(in_D&gt;0,in_D&amp;" x D (4 MP)  ","")&amp;IF(in_NP&gt;0,in_NP&amp;" x N.P.  ","")&amp;"= "&amp;m_MP&amp;" MP"</f>
@@ -3207,7 +3210,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C44" s="16" t="str">
         <f aca="false">IF(t_zaglebienia="","standard 170 cm",t_zaglebienia)</f>
@@ -3221,7 +3224,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C45" s="16" t="str">
         <f aca="false">IF(t_wymiary="","standard",t_wymiary)</f>
@@ -3235,7 +3238,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C46" s="16" t="str">
         <f aca="false">in_magistrala&amp;" x 6 m  /  "&amp;in_barierki&amp;" szt.  /  "&amp;in_maskownice&amp;" szt."</f>
@@ -3249,7 +3252,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C47" s="16" t="str">
         <f aca="false">m_utr&amp;" (z magistrali i barierek "&amp;m_utr_auto&amp;", ręcznie "&amp;in_utr_dod&amp;")"</f>
@@ -3277,7 +3280,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C49" s="16" t="str">
         <f aca="false">e_km_pom&amp;" / "&amp;e_km_mon&amp;" km"</f>
@@ -3291,11 +3294,11 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C50" s="16" t="str">
-        <f aca="false">in_tir&amp;" TIR x "&amp;TEXT(in_tir_cena,"#,##0")&amp;" zł, rozładunek "&amp;TEXT(in_rozl_cena,"#,##0")&amp;" zł/TIR, "&amp;e_rozl_dni&amp;" dni"</f>
-        <v>0 TIR x 0 zł, rozładunek 0 zł/TIR, 0 dni</v>
+        <f aca="false">in_tir&amp;" TIR x "&amp;TEXT(in_tir_cena,"#,##0")&amp;" zł, rozładunek sprzętu "&amp;TEXT(in_rozl_cena,"#,##0")&amp;" zł jednorazowo, "&amp;e_rozl_dni&amp;" dni"</f>
+        <v>0 TIR x 0 zł, rozładunek sprzętu 0 zł jednorazowo, 0 dni</v>
       </c>
       <c r="D50" s="16"/>
       <c r="E50" s="16"/>
@@ -3305,7 +3308,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C51" s="16" t="str">
         <f aca="false">in_osoby&amp;" osób, średnia stawka "&amp;TEXT(Obliczenia!D41,"#,##0")&amp;" zł/dzień"</f>
@@ -3319,7 +3322,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C52" s="16" t="str">
         <f aca="false">e_dzw_dni&amp;" dni"</f>
@@ -3333,7 +3336,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="0" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C53" s="16" t="str">
         <f aca="false">Obliczenia!D51&amp;" dni pracy = "&amp;Obliczenia!D48&amp;IF(e_krk," dni"," tyg.")&amp;", "&amp;TEXT(Obliczenia!D50,"0.0")&amp;" osobodni"</f>
@@ -3347,7 +3350,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="0" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C54" s="16" t="str">
         <f aca="false">Obliczenia!F51&amp;" dni pracy = "&amp;Obliczenia!F48&amp;IF(e_krk," dni"," tyg.")&amp;", "&amp;TEXT(Obliczenia!F50,"0.0")&amp;" osobodni"</f>
@@ -3361,7 +3364,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C55" s="16" t="str">
         <f aca="false">TEXT(in_zysk,"0.0%")&amp;" / "&amp;TEXT(in_zysk2,"0.0%")</f>
@@ -3375,7 +3378,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C56" s="16" t="str">
         <f aca="false">TEXT(in_q2500,"0.0%")</f>
@@ -3403,11 +3406,11 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C58" s="16" t="str">
-        <f aca="false">TEXT(c_konserw*m_MP*12,"#,##0")&amp;" / "&amp;TEXT(c_konserw2*m_MP*12,"#,##0")&amp;" / "&amp;TEXT(c_konserw3*m_MP*12,"#,##0")&amp;" zł"</f>
-        <v>0 / 0 / 0 zł</v>
+        <f aca="false">TEXT(in_konsA*m_MP*12,"#,##0")&amp;" / "&amp;TEXT(in_konsB*m_MP*12,"#,##0")&amp;" zł  (przegląd półroczny "&amp;TEXT(in_konsA*m_MP*6,"#,##0")&amp;" / "&amp;TEXT(in_konsB*m_MP*6,"#,##0")&amp;" zł)"</f>
+        <v>0 / 0 zł  (przegląd półroczny 0 / 0 zł)</v>
       </c>
       <c r="D58" s="16"/>
       <c r="E58" s="16"/>
@@ -3417,7 +3420,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C59" s="16" t="str">
         <f aca="false">in_opis&amp;""</f>
@@ -3431,16 +3434,16 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="11" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C61" s="0" t="str">
-        <f aca="false">IF(COUNTIF(Dane!B63:B68,"ok")=6,"wszystko ok","sprawdź arkusz Dane")</f>
+        <f aca="false">IF(COUNTIF(Dane!B65:B70,"ok")=6,"wszystko ok","sprawdź arkusz Dane")</f>
         <v>sprawdź arkusz Dane</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C63" s="5"/>
       <c r="D63" s="5"/>
@@ -3451,7 +3454,7 @@
     </row>
     <row r="64" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="24" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C64" s="24"/>
       <c r="D64" s="24"/>
@@ -3462,7 +3465,7 @@
     </row>
     <row r="65" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="24" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C65" s="24"/>
       <c r="D65" s="24"/>
@@ -3473,7 +3476,7 @@
     </row>
     <row r="66" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B66" s="24" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C66" s="24"/>
       <c r="D66" s="24"/>
@@ -3484,7 +3487,7 @@
     </row>
     <row r="67" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="24" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C67" s="24"/>
       <c r="D67" s="24"/>
@@ -3495,7 +3498,7 @@
     </row>
     <row r="68" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="24" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C68" s="24"/>
       <c r="D68" s="24"/>
@@ -3504,8 +3507,19 @@
       <c r="G68" s="24"/>
       <c r="H68" s="24"/>
     </row>
+    <row r="69" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B69" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="C69" s="24"/>
+      <c r="D69" s="24"/>
+      <c r="E69" s="24"/>
+      <c r="F69" s="24"/>
+      <c r="G69" s="24"/>
+      <c r="H69" s="24"/>
+    </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="24">
     <mergeCell ref="C42:H42"/>
     <mergeCell ref="C43:H43"/>
     <mergeCell ref="C44:H44"/>
@@ -3529,6 +3543,7 @@
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B67:H67"/>
     <mergeCell ref="B68:H68"/>
+    <mergeCell ref="B69:H69"/>
   </mergeCells>
   <conditionalFormatting sqref="C34:H34">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
@@ -3555,7 +3570,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:F113"/>
+  <dimension ref="B2:F109"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -3567,7 +3582,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -3576,12 +3591,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -3589,90 +3604,90 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="0" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>32500</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="0" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>700</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="0" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>0.61</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="0" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C9" s="14" t="n">
         <v>0.85</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="0" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1170</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="0" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1560</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="0" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1820</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="0" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>3110</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3683,34 +3698,34 @@
         <v>2340</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="0" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C15" s="25" t="n">
         <v>0.00127</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="0" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C16" s="14" t="n">
         <v>0.07</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="4" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
@@ -3718,107 +3733,107 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="0" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>6500</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="0" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1500</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="0" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>200</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="0" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>500</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="0" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>50</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1080</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="0" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1175</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="0" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1250</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="0" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C26" s="26" t="n">
         <f aca="false">0.2*11+0.4*11+2*14+6*11+6*5+6*10</f>
         <v>190.6</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -3826,51 +3841,51 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="0" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>600</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="0" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>700</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="0" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1000</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="0" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1800</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="4" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
@@ -3878,73 +3893,73 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="0" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>6400</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>13500</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="0" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>200</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="0" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1700</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="0" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>6300</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="0" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C38" s="9" t="n">
         <v>0.37</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="4" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
@@ -3952,117 +3967,117 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="0" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="C40" s="9" t="n">
         <v>5.5</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="0" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C41" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="0" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C42" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C43" s="9" t="n">
         <v>0.5</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="0" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C44" s="9" t="n">
         <v>0.5</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="0" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C45" s="9" t="n">
         <v>0.5</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="0" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>2400</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="0" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C47" s="9" t="n">
         <v>5</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="0" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C48" s="9" t="n">
         <v>0.6</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C49" s="9" t="n">
         <v>5</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="4" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5"/>
@@ -4070,84 +4085,84 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="0" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C51" s="9" t="n">
         <v>50</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C52" s="9" t="n">
         <v>20</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="0" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C53" s="9" t="n">
         <v>650</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="0" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C54" s="9" t="n">
         <v>12</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="0" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="C55" s="26" t="n">
         <v>9.4</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="0" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="C56" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C57" s="9" t="n">
         <v>2</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="4" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5"/>
@@ -4155,62 +4170,62 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="0" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>500</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>400</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C61" s="13" t="n">
         <v>350</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C62" s="13" t="n">
         <v>45</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C63" s="13" t="n">
         <v>130</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C64" s="5"/>
       <c r="D64" s="5"/>
@@ -4218,103 +4233,106 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="0" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C65" s="14" t="n">
         <v>0.005</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="0" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C66" s="14" t="n">
         <v>0.025</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="0" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="C67" s="14" t="n">
         <v>0.14</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B68" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="C68" s="5"/>
-      <c r="D68" s="5"/>
-      <c r="E68" s="5"/>
+        <v>251</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B69" s="0" t="s">
-        <v>250</v>
-      </c>
-      <c r="C69" s="13" t="n">
-        <v>40</v>
-      </c>
-      <c r="E69" s="8" t="s">
-        <v>251</v>
-      </c>
+      <c r="B69" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C69" s="5"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B70" s="0" t="s">
-        <v>252</v>
-      </c>
-      <c r="C70" s="13" t="n">
-        <v>45</v>
-      </c>
-      <c r="E70" s="8" t="s">
+      <c r="B70" s="11" t="s">
         <v>253</v>
       </c>
+      <c r="C70" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="D70" s="11" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B71" s="0" t="s">
-        <v>254</v>
-      </c>
-      <c r="C71" s="13" t="n">
-        <v>50</v>
-      </c>
-      <c r="E71" s="8" t="s">
-        <v>255</v>
+      <c r="B71" s="0" t="n">
+        <v>175</v>
+      </c>
+      <c r="C71" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="28" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B72" s="0" t="n">
+        <v>180</v>
+      </c>
+      <c r="C72" s="27" t="n">
+        <v>500</v>
+      </c>
+      <c r="D72" s="28" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B73" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="C73" s="5"/>
-      <c r="D73" s="5"/>
-      <c r="E73" s="5"/>
+      <c r="B73" s="0" t="n">
+        <v>185</v>
+      </c>
+      <c r="C73" s="27" t="n">
+        <v>550</v>
+      </c>
+      <c r="D73" s="28" t="n">
+        <v>2000</v>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B74" s="11" t="s">
-        <v>257</v>
-      </c>
-      <c r="C74" s="11" t="s">
-        <v>258</v>
-      </c>
-      <c r="D74" s="11" t="s">
-        <v>259</v>
+      <c r="B74" s="0" t="n">
+        <v>190</v>
+      </c>
+      <c r="C74" s="27" t="n">
+        <v>600</v>
+      </c>
+      <c r="D74" s="28" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="0" t="n">
-        <v>175</v>
+        <v>195</v>
       </c>
       <c r="C75" s="27" t="n">
-        <v>0</v>
+        <v>650</v>
       </c>
       <c r="D75" s="28" t="n">
         <v>2000</v>
@@ -4322,10 +4340,10 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="0" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C76" s="27" t="n">
-        <v>500</v>
+        <v>700</v>
       </c>
       <c r="D76" s="28" t="n">
         <v>2000</v>
@@ -4333,122 +4351,146 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="0" t="n">
-        <v>185</v>
+        <v>210</v>
       </c>
       <c r="C77" s="27" t="n">
-        <v>550</v>
+        <v>750</v>
       </c>
       <c r="D77" s="28" t="n">
-        <v>2000</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="0" t="n">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="C78" s="27" t="n">
-        <v>600</v>
+        <v>800</v>
       </c>
       <c r="D78" s="28" t="n">
-        <v>2000</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="0" t="n">
-        <v>195</v>
+        <v>225</v>
       </c>
       <c r="C79" s="27" t="n">
-        <v>650</v>
+        <v>850</v>
       </c>
       <c r="D79" s="28" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B80" s="0" t="n">
-        <v>200</v>
-      </c>
-      <c r="C80" s="27" t="n">
-        <v>700</v>
-      </c>
-      <c r="D80" s="28" t="n">
-        <v>2000</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B81" s="0" t="n">
-        <v>210</v>
-      </c>
-      <c r="C81" s="27" t="n">
-        <v>750</v>
-      </c>
-      <c r="D81" s="28" t="n">
-        <v>2250</v>
-      </c>
+      <c r="B81" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C81" s="5"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
+      <c r="F81" s="5"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B82" s="0" t="n">
-        <v>220</v>
-      </c>
-      <c r="C82" s="27" t="n">
-        <v>800</v>
-      </c>
-      <c r="D82" s="28" t="n">
-        <v>2250</v>
+      <c r="B82" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="C82" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="D82" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="E82" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="F82" s="11" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B83" s="0" t="n">
-        <v>225</v>
-      </c>
-      <c r="C83" s="27" t="n">
-        <v>850</v>
+      <c r="B83" s="0" t="s">
+        <v>262</v>
+      </c>
+      <c r="C83" s="29" t="n">
+        <v>45</v>
       </c>
       <c r="D83" s="28" t="n">
-        <v>2250</v>
+        <v>9.6</v>
+      </c>
+      <c r="E83" s="28" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F83" s="30" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B84" s="0" t="s">
+        <v>264</v>
+      </c>
+      <c r="C84" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="D84" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="E84" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="F84" s="30" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B85" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="C85" s="5"/>
-      <c r="D85" s="5"/>
-      <c r="E85" s="5"/>
-      <c r="F85" s="5"/>
+      <c r="B85" s="0" t="s">
+        <v>265</v>
+      </c>
+      <c r="C85" s="29" t="n">
+        <v>36</v>
+      </c>
+      <c r="D85" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E85" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" s="30" t="s">
+        <v>263</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B86" s="11" t="s">
-        <v>261</v>
-      </c>
-      <c r="C86" s="11" t="s">
-        <v>262</v>
-      </c>
-      <c r="D86" s="11" t="s">
+      <c r="B86" s="0" t="s">
+        <v>266</v>
+      </c>
+      <c r="C86" s="29" t="n">
+        <v>90</v>
+      </c>
+      <c r="D86" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E86" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F86" s="30" t="s">
         <v>263</v>
-      </c>
-      <c r="E86" s="11" t="s">
-        <v>264</v>
-      </c>
-      <c r="F86" s="11" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="0" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C87" s="29" t="n">
-        <v>45</v>
+        <v>207.28</v>
       </c>
       <c r="D87" s="28" t="n">
-        <v>9.6</v>
+        <v>2</v>
       </c>
       <c r="E87" s="28" t="n">
-        <v>9.6</v>
+        <v>2</v>
       </c>
       <c r="F87" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4456,16 +4498,16 @@
         <v>268</v>
       </c>
       <c r="C88" s="29" t="n">
-        <v>8</v>
+        <v>40.14</v>
       </c>
       <c r="D88" s="28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E88" s="28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F88" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4473,7 +4515,7 @@
         <v>269</v>
       </c>
       <c r="C89" s="29" t="n">
-        <v>36</v>
+        <v>3.3</v>
       </c>
       <c r="D89" s="28" t="n">
         <v>2</v>
@@ -4482,7 +4524,7 @@
         <v>2</v>
       </c>
       <c r="F89" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4490,7 +4532,7 @@
         <v>270</v>
       </c>
       <c r="C90" s="29" t="n">
-        <v>90</v>
+        <v>10.8</v>
       </c>
       <c r="D90" s="28" t="n">
         <v>2</v>
@@ -4499,7 +4541,7 @@
         <v>2</v>
       </c>
       <c r="F90" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4507,7 +4549,7 @@
         <v>271</v>
       </c>
       <c r="C91" s="29" t="n">
-        <v>207.28</v>
+        <v>10.95</v>
       </c>
       <c r="D91" s="28" t="n">
         <v>2</v>
@@ -4516,7 +4558,7 @@
         <v>2</v>
       </c>
       <c r="F91" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4524,7 +4566,7 @@
         <v>272</v>
       </c>
       <c r="C92" s="29" t="n">
-        <v>40.14</v>
+        <v>3.81</v>
       </c>
       <c r="D92" s="28" t="n">
         <v>2</v>
@@ -4533,7 +4575,7 @@
         <v>2</v>
       </c>
       <c r="F92" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4541,16 +4583,16 @@
         <v>273</v>
       </c>
       <c r="C93" s="29" t="n">
-        <v>3.3</v>
+        <v>2.84</v>
       </c>
       <c r="D93" s="28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E93" s="28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F93" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4558,16 +4600,16 @@
         <v>274</v>
       </c>
       <c r="C94" s="29" t="n">
-        <v>10.8</v>
+        <v>4.4</v>
       </c>
       <c r="D94" s="28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E94" s="28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F94" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4575,16 +4617,17 @@
         <v>275</v>
       </c>
       <c r="C95" s="29" t="n">
-        <v>10.95</v>
+        <f aca="false">2*25.71+2*22.85</f>
+        <v>97.12</v>
       </c>
       <c r="D95" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E95" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F95" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4592,16 +4635,16 @@
         <v>276</v>
       </c>
       <c r="C96" s="29" t="n">
-        <v>3.81</v>
+        <v>345</v>
       </c>
       <c r="D96" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E96" s="28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F96" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4609,16 +4652,16 @@
         <v>277</v>
       </c>
       <c r="C97" s="29" t="n">
-        <v>2.84</v>
+        <v>546</v>
       </c>
       <c r="D97" s="28" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E97" s="28" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F97" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4626,16 +4669,16 @@
         <v>278</v>
       </c>
       <c r="C98" s="29" t="n">
-        <v>4.4</v>
+        <v>2.98</v>
       </c>
       <c r="D98" s="28" t="n">
-        <v>4</v>
+        <v>110</v>
       </c>
       <c r="E98" s="28" t="n">
-        <v>4</v>
+        <v>208</v>
       </c>
       <c r="F98" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4643,17 +4686,17 @@
         <v>279</v>
       </c>
       <c r="C99" s="29" t="n">
-        <f aca="false">2*25.71+2*22.85</f>
-        <v>97.12</v>
+        <f aca="false">3.09+4.99</f>
+        <v>8.08</v>
       </c>
       <c r="D99" s="28" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E99" s="28" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F99" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4661,16 +4704,16 @@
         <v>280</v>
       </c>
       <c r="C100" s="29" t="n">
-        <v>345</v>
+        <v>5.4</v>
       </c>
       <c r="D100" s="28" t="n">
         <v>1</v>
       </c>
       <c r="E100" s="28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F100" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4678,16 +4721,16 @@
         <v>281</v>
       </c>
       <c r="C101" s="29" t="n">
-        <v>546</v>
+        <v>300</v>
       </c>
       <c r="D101" s="28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E101" s="28" t="n">
         <v>1</v>
       </c>
       <c r="F101" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4695,16 +4738,16 @@
         <v>282</v>
       </c>
       <c r="C102" s="29" t="n">
-        <v>2.98</v>
+        <v>40</v>
       </c>
       <c r="D102" s="28" t="n">
-        <v>110</v>
+        <v>1</v>
       </c>
       <c r="E102" s="28" t="n">
-        <v>208</v>
+        <v>1</v>
       </c>
       <c r="F102" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4712,17 +4755,16 @@
         <v>283</v>
       </c>
       <c r="C103" s="29" t="n">
-        <f aca="false">3.09+4.99</f>
-        <v>8.08</v>
+        <v>172</v>
       </c>
       <c r="D103" s="28" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E103" s="28" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F103" s="30" t="s">
-        <v>267</v>
+        <v>162</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4730,16 +4772,16 @@
         <v>284</v>
       </c>
       <c r="C104" s="29" t="n">
-        <v>5.4</v>
+        <v>207</v>
       </c>
       <c r="D104" s="28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E104" s="28" t="n">
         <v>1</v>
       </c>
       <c r="F104" s="30" t="s">
-        <v>267</v>
+        <v>162</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4747,7 +4789,8 @@
         <v>285</v>
       </c>
       <c r="C105" s="29" t="n">
-        <v>300</v>
+        <f aca="false">120+55+65</f>
+        <v>240</v>
       </c>
       <c r="D105" s="28" t="n">
         <v>1</v>
@@ -4756,7 +4799,7 @@
         <v>1</v>
       </c>
       <c r="F105" s="30" t="s">
-        <v>267</v>
+        <v>162</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4764,7 +4807,8 @@
         <v>286</v>
       </c>
       <c r="C106" s="29" t="n">
-        <v>40</v>
+        <f aca="false">50+40</f>
+        <v>90</v>
       </c>
       <c r="D106" s="28" t="n">
         <v>1</v>
@@ -4773,32 +4817,34 @@
         <v>1</v>
       </c>
       <c r="F106" s="30" t="s">
-        <v>267</v>
+        <v>287</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B107" s="0" t="s">
+        <v>288</v>
+      </c>
+      <c r="C107" s="29" t="n">
+        <f aca="false">14+9+25+5+9+30</f>
+        <v>92</v>
+      </c>
+      <c r="D107" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" s="30" t="s">
         <v>287</v>
-      </c>
-      <c r="C107" s="29" t="n">
-        <v>172</v>
-      </c>
-      <c r="D107" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E107" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F107" s="30" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B108" s="0" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C108" s="29" t="n">
-        <v>207</v>
+        <f aca="false">14+18+25+7+18+30</f>
+        <v>112</v>
       </c>
       <c r="D108" s="28" t="n">
         <v>0</v>
@@ -4807,97 +4853,25 @@
         <v>1</v>
       </c>
       <c r="F108" s="30" t="s">
-        <v>159</v>
+        <v>287</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="0" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C109" s="29" t="n">
-        <f aca="false">120+55+65</f>
-        <v>240</v>
-      </c>
-      <c r="D109" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E109" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F109" s="30" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B110" s="0" t="s">
-        <v>290</v>
-      </c>
-      <c r="C110" s="29" t="n">
-        <f aca="false">50+40</f>
-        <v>90</v>
-      </c>
-      <c r="D110" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E110" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F110" s="30" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B111" s="0" t="s">
-        <v>292</v>
-      </c>
-      <c r="C111" s="29" t="n">
-        <f aca="false">14+9+25+5+9+30</f>
-        <v>92</v>
-      </c>
-      <c r="D111" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E111" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F111" s="30" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B112" s="0" t="s">
-        <v>293</v>
-      </c>
-      <c r="C112" s="29" t="n">
-        <f aca="false">14+18+25+7+18+30</f>
-        <v>112</v>
-      </c>
-      <c r="D112" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E112" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F112" s="30" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B113" s="0" t="s">
-        <v>294</v>
-      </c>
-      <c r="C113" s="29" t="n">
         <f aca="false">70+14+34+32+20</f>
         <v>170</v>
       </c>
-      <c r="D113" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E113" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F113" s="30" t="s">
-        <v>291</v>
+      <c r="D109" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" s="30" t="s">
+        <v>287</v>
       </c>
     </row>
   </sheetData>
@@ -4928,7 +4902,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -4945,13 +4919,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="C4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="0" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="C5" s="31" t="n">
         <f aca="false">c_cena_D+IF(in_typ="NK37",c_doplata_NK37,0)</f>
@@ -4960,7 +4934,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="0" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="C6" s="31" t="n">
         <f aca="false">c_wsp_S*m_cena_D</f>
@@ -4969,7 +4943,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="0" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="C7" s="31" t="n">
         <f aca="false">c_wsp_NP*m_cena_D</f>
@@ -4978,7 +4952,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="0" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="C8" s="32" t="n">
         <f aca="false">in_D+in_NP</f>
@@ -4987,7 +4961,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="0" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="C9" s="32" t="n">
         <f aca="false">in_S+in_D+in_NP</f>
@@ -4996,7 +4970,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="0" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="C10" s="32" t="n">
         <f aca="false">2*in_S+2*in_NP+4*in_D</f>
@@ -5005,7 +4979,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="0" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="C11" s="31" t="n">
         <f aca="false">m_cena_S*in_S+c_szer_260*in_szer1_S+c_szer_270*in_szer2_S+SUMPRODUCT(in_gl_S,t_gl_doplata)+c_dl_500*in_dl500_S+CEILING(m_cena_S*c_dl_wsp*10,100)*in_dl540_S+CEILING(m_cena_S*c_dl_wsp*20,100)*in_dl550_S</f>
@@ -5014,7 +4988,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="0" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="C12" s="31" t="n">
         <f aca="false">m_cena_D*in_D+c_szer_520*in_szer1_D+c_szer_540*in_szer2_D+SUMPRODUCT(in_gl_D,t_gl_doplata)+c_dl_500*in_dl500_D+m_cena_D*c_dl_wsp*10*in_dl540_D+m_cena_D*c_dl_wsp*20*in_dl550_D</f>
@@ -5023,7 +4997,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="0" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="C13" s="31" t="n">
         <f aca="false">m_cena_NP*in_NP</f>
@@ -5032,7 +5006,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="0" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="C14" s="32" t="n">
         <f aca="false">SUMPRODUCT((t_gl_silownik=2000)*(in_gl_S+in_gl_D))</f>
@@ -5041,7 +5015,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="0" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="C15" s="32" t="n">
         <f aca="false">SUMPRODUCT((t_gl_silownik=2250)*(in_gl_S+in_gl_D))</f>
@@ -5050,7 +5024,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="0" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="C16" s="32" t="n">
         <f aca="false">m_platformy-m_sil_2000-m_sil_2250</f>
@@ -5059,7 +5033,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C17" s="31" t="n">
         <f aca="false">in_agregaty*(c_agregat+c_hydr_drobne+c_olej+c_transp_agregatu)+m_platformy*c_transp_silownikow+2*(c_sil_1700*m_sil_std+c_sil_2000*m_sil_2000+c_sil_2250*m_sil_2250)+in_magistrala*c_magistrala+SUMPRODUCT((t_sk_grupa="Hydraulika")*t_sk_cena*(t_sk_S*in_S+t_sk_D*m_DN))</f>
@@ -5068,7 +5042,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="0" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="C18" s="31" t="n">
         <f aca="false">in_barierki*c_barierka+in_maskownice*c_maskownica</f>
@@ -5077,7 +5051,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="0" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C19" s="31" t="n">
         <f aca="false">in_agregaty*c_skrzynka_zasil+SUMPRODUCT((t_sk_grupa="Elektryka")*t_sk_cena*(t_sk_S*in_S+t_sk_D*m_DN))</f>
@@ -5086,7 +5060,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="0" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="C20" s="31" t="n">
         <f aca="false">in_agregaty*c_admin+SUMPRODUCT((t_sk_grupa="Mechanika")*t_sk_cena*(t_sk_S*in_S+t_sk_D*m_DN))</f>
@@ -5095,7 +5069,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="11" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C21" s="33" t="n">
         <f aca="false">m_plat_S+m_plat_D+m_plat_NP+m_hydraulika+m_barierki+m_elektryka+m_mechanika</f>
@@ -5104,7 +5078,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="11" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C22" s="33" t="n">
         <f aca="false">m_suma_2000*(1+in_q2500)</f>
@@ -5113,7 +5087,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="0" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="C23" s="31" t="n">
         <f aca="false">c_mal_S*in_S+c_mal_D*m_DN+c_mal_bar*in_barierki</f>
@@ -5122,7 +5096,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="0" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="C24" s="34" t="n">
         <f aca="false">ROUNDUP(in_magistrala*c_osd_magistrala+(in_barierki+in_maskownice)*c_osd_barierka,0)</f>
@@ -5131,7 +5105,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="0" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="C25" s="34" t="n">
         <f aca="false">m_utr_auto+in_utr_dod</f>
@@ -5140,13 +5114,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="C27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="0" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="C28" s="35" t="b">
         <f aca="false">in_lok="Kraków"</f>
@@ -5155,7 +5129,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="0" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="C29" s="34" t="n">
         <f aca="false">IF(ISBLANK(in_km_pom),IF(e_krk,c_km_krakow,in_km),in_km_pom)</f>
@@ -5164,7 +5138,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="0" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="C30" s="34" t="n">
         <f aca="false">IF(ISBLANK(in_km_mon),IF(e_krk,c_km_krakow,in_km+c_km_dodatek),in_km_mon)</f>
@@ -5173,7 +5147,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="0" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C31" s="34" t="n">
         <f aca="false">IF(ISBLANK(in_rozl_dni),c_rozl_TIR*in_tir,in_rozl_dni)</f>
@@ -5182,7 +5156,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="0" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="C32" s="34" t="n">
         <f aca="false">(c_pomiary_osoby+c_odbiory_osoby)*IF(in_wzor="Uproszczony",2*e_km_pom/c_km_dzien*1,(1+0.1*MAX(0,800-e_km_pom)/100)*e_km_pom*1/500)</f>
@@ -5191,7 +5165,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="0" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="C33" s="32" t="n">
         <f aca="false">ROUNDUP(m_DN/c_dzwig_D+in_S*c_dzwig_wspS/c_dzwig_D,0)</f>
@@ -5200,7 +5174,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="C34" s="36" t="n">
         <f aca="false">(1+c_podatek*(c_gdw+in_zysk))/(1-(c_kob+c_gdw+in_zysk))</f>
@@ -5209,7 +5183,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="4" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
@@ -5218,7 +5192,7 @@
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
       <c r="I36" s="4" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="J36" s="5"/>
       <c r="K36" s="5"/>
@@ -5228,42 +5202,42 @@
     </row>
     <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="11" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="D37" s="37" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E37" s="37" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F37" s="37" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G37" s="37" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I37" s="37" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="J37" s="37" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K37" s="37" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="L37" s="37" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="M37" s="37" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="N37" s="37" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="0" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="D38" s="32" t="n">
         <v>0</v>
@@ -5304,7 +5278,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="0" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D39" s="32" t="n">
         <v>0</v>
@@ -5345,7 +5319,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="0" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D40" s="32" t="n">
         <f aca="false">in_osoby</f>
@@ -5384,7 +5358,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="0" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="D41" s="31" t="n">
         <f aca="false">(c_stawka_1+IF(D40&gt;=2,c_stawka_2,0)+MAX(0,D40-2)*c_stawka_n)/D40</f>
@@ -5429,7 +5403,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="0" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="D42" s="34" t="n">
         <f aca="false">c_osd_S*in_S+c_osd_D*in_D+c_osd_NP*in_NP+m_utr+D39*c_slupek_rbd*m_MP</f>
@@ -5474,7 +5448,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="0" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="D43" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*1,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*1/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*1,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*1/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5519,7 +5493,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="0" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="D44" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D43,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D43/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D43,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D43/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5564,7 +5538,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="0" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="D45" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D44,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D44/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D44,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D44/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5609,7 +5583,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="0" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="D46" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D45,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D45/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D45,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D45/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5654,7 +5628,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="0" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="D47" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D46,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D46/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D46,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D46/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5699,7 +5673,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="11" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="D48" s="38" t="n">
         <f aca="false">IF(ISBLANK(in_wyjazdy),D47,in_wyjazdy)</f>
@@ -5744,7 +5718,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="0" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="D49" s="34" t="n">
         <f aca="false">(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D48,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D48/500)))</f>
@@ -5789,7 +5763,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="0" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D50" s="34" t="n">
         <f aca="false">D42+D49</f>
@@ -5834,7 +5808,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="11" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="D51" s="38" t="n">
         <f aca="false">CEILING(D50/D40,1)</f>
@@ -5879,7 +5853,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="11" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="D52" s="38" t="n">
         <f aca="false">IF(e_krk,CEILING(D51/c_dni_tydzien,1),D48)</f>
@@ -5924,7 +5898,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="0" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="D53" s="34" t="n">
         <f aca="false">2*(e_km_mon*D48+2*e_km_pom)</f>
@@ -5969,7 +5943,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D54" s="31" t="n">
         <f aca="false">IF(D38=1,m_suma_2500,m_suma_2000)</f>
@@ -6014,7 +5988,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="0" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D55" s="31" t="n">
         <f aca="false">D39*c_slupek*m_MP</f>
@@ -6059,7 +6033,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="0" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="D56" s="31" t="n">
         <f aca="false">D53/100*ROUNDUP(c_spalanie*c_paliwo,0)</f>
@@ -6104,7 +6078,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="0" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="D57" s="31" t="n">
         <f aca="false">IF(e_krk,0,c_hotel*(D51+1)*D40)</f>
@@ -6149,7 +6123,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="0" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="D58" s="31" t="n">
         <f aca="false">in_tir_cena*in_tir</f>
@@ -6194,7 +6168,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="0" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="D59" s="31" t="n">
         <f aca="false">c_dzwig*e_dzw_dni</f>
@@ -6239,52 +6213,52 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="0" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="D60" s="31" t="n">
-        <f aca="false">in_rozl_cena*in_tir</f>
+        <f aca="false">in_rozl_cena</f>
         <v>0</v>
       </c>
       <c r="E60" s="31" t="n">
-        <f aca="false">in_rozl_cena*in_tir</f>
+        <f aca="false">in_rozl_cena</f>
         <v>0</v>
       </c>
       <c r="F60" s="31" t="n">
-        <f aca="false">in_rozl_cena*in_tir</f>
+        <f aca="false">in_rozl_cena</f>
         <v>0</v>
       </c>
       <c r="G60" s="31" t="n">
-        <f aca="false">in_rozl_cena*in_tir</f>
+        <f aca="false">in_rozl_cena</f>
         <v>0</v>
       </c>
       <c r="I60" s="31" t="n">
-        <f aca="false">in_rozl_cena*in_tir</f>
+        <f aca="false">in_rozl_cena</f>
         <v>0</v>
       </c>
       <c r="J60" s="31" t="n">
-        <f aca="false">in_rozl_cena*in_tir</f>
+        <f aca="false">in_rozl_cena</f>
         <v>0</v>
       </c>
       <c r="K60" s="31" t="n">
-        <f aca="false">in_rozl_cena*in_tir</f>
+        <f aca="false">in_rozl_cena</f>
         <v>0</v>
       </c>
       <c r="L60" s="31" t="n">
-        <f aca="false">in_rozl_cena*in_tir</f>
+        <f aca="false">in_rozl_cena</f>
         <v>0</v>
       </c>
       <c r="M60" s="31" t="n">
-        <f aca="false">in_rozl_cena*in_tir</f>
+        <f aca="false">in_rozl_cena</f>
         <v>0</v>
       </c>
       <c r="N60" s="31" t="n">
-        <f aca="false">in_rozl_cena*in_tir</f>
+        <f aca="false">in_rozl_cena</f>
         <v>0</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="0" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="D61" s="31" t="n">
         <f aca="false">D41*e_rozl_dni*D40</f>
@@ -6329,7 +6303,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="0" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="D62" s="31" t="n">
         <f aca="false">D41*(D49-D40*e_rozl_dni)</f>
@@ -6374,7 +6348,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="0" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="D63" s="31" t="n">
         <f aca="false">IF(D48&gt;0,D41*D42,0)</f>
@@ -6419,7 +6393,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="0" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="D64" s="31" t="n">
         <f aca="false">IF(e_krk,0,c_dieta*D50)</f>
@@ -6464,7 +6438,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="11" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="D65" s="33" t="n">
         <f aca="false">SUM(D54:D64)</f>
@@ -6509,7 +6483,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="0" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="D66" s="31" t="n">
         <f aca="false">D65/(1-(c_kob+c_gdw+in_zysk))</f>
@@ -6554,7 +6528,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="0" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="D67" s="31" t="n">
         <f aca="false">D66*c_kob</f>
@@ -6599,7 +6573,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="0" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="D68" s="31" t="n">
         <f aca="false">D66*c_gdw</f>
@@ -6644,7 +6618,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="0" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="D69" s="31" t="n">
         <f aca="false">D66*in_zysk</f>
@@ -6689,7 +6663,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="0" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="D70" s="31" t="n">
         <f aca="false">c_podatek*(D61+D62+D63+D64+D68+D69)</f>
@@ -6734,7 +6708,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="11" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="D71" s="33" t="n">
         <f aca="false">D66+D70</f>
@@ -6779,7 +6753,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="0" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="D72" s="31" t="n">
         <f aca="false">D71-D69</f>
@@ -6824,7 +6798,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D73" s="31" t="n">
         <f aca="false">IF(m_MP&gt;0,D71/m_MP,0)</f>
@@ -6869,7 +6843,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="0" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="D74" s="39" t="n">
         <f aca="false">D73/in_eur</f>
@@ -6914,7 +6888,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="0" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="D75" s="31" t="n">
         <f aca="false">D65/(1-(c_kob+c_gdw+in_zysk2))</f>
@@ -6959,7 +6933,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="0" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="D76" s="31" t="n">
         <f aca="false">D75*in_zysk2</f>
@@ -7004,7 +6978,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="11" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="D77" s="33" t="n">
         <f aca="false">D75+c_podatek*(D61+D62+D63+D64+D75*(c_gdw+in_zysk2))</f>
@@ -7049,7 +7023,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D78" s="31" t="n">
         <f aca="false">IF(m_MP&gt;0,D77/m_MP,0)</f>

</xml_diff>

<commit_message>
NK38: panel oferty, edytor szablonów urządzeń, baza danych strony
- oferta jako osobny panel pod pulpitem: sekcje z adresatem, specyfikacją, cenami, tekstami stałymi, podpisem i logo, podgląd na żywo
- zakładka Szablony urządzeń: edycja typów, cennika, zagłębień, wymiarów i składowych, kopia, eksport i import
- opis wariantu tworzony automatycznie, cena dźwigu za dzień pod polem
- stawki konserwacji przy wynikach, zysk jako procent
- usunięte przykłady i zakładka Uwagi, poprawione przewijanie
- przegenerowany Excel z ręcznym kosztem dźwigu

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/Kalkulator_NK38_v1.xlsx
+++ b/kalkulator-nk38/Kalkulator_NK38_v1.xlsx
@@ -77,7 +77,7 @@
     <definedName function="false" hidden="false" name="e_podr_pom" vbProcedure="false">Obliczenia!$C$32</definedName>
     <definedName function="false" hidden="false" name="e_rozl_dni" vbProcedure="false">Obliczenia!$C$31</definedName>
     <definedName function="false" hidden="false" name="in_agregaty" vbProcedure="false">Dane!$C$22</definedName>
-    <definedName function="false" hidden="false" name="in_analiza" vbProcedure="false">Dane!$C$62</definedName>
+    <definedName function="false" hidden="false" name="in_analiza" vbProcedure="false">Dane!$C$63</definedName>
     <definedName function="false" hidden="false" name="in_barierki" vbProcedure="false">Dane!$C$24</definedName>
     <definedName function="false" hidden="false" name="in_D" vbProcedure="false">Dane!$C$20</definedName>
     <definedName function="false" hidden="false" name="in_data" vbProcedure="false">Dane!$C$7</definedName>
@@ -87,14 +87,15 @@
     <definedName function="false" hidden="false" name="in_dl540_S" vbProcedure="false">Dane!$C$43</definedName>
     <definedName function="false" hidden="false" name="in_dl550_D" vbProcedure="false">Dane!$D$44</definedName>
     <definedName function="false" hidden="false" name="in_dl550_S" vbProcedure="false">Dane!$C$44</definedName>
-    <definedName function="false" hidden="false" name="in_eur" vbProcedure="false">Dane!$C$59</definedName>
+    <definedName function="false" hidden="false" name="in_dzwig_koszt" vbProcedure="false">Dane!$C$51</definedName>
+    <definedName function="false" hidden="false" name="in_eur" vbProcedure="false">Dane!$C$60</definedName>
     <definedName function="false" hidden="false" name="in_gl_D" vbProcedure="false">Dane!$D$30:$D$38</definedName>
     <definedName function="false" hidden="false" name="in_gl_S" vbProcedure="false">Dane!$C$30:$C$38</definedName>
     <definedName function="false" hidden="false" name="in_km" vbProcedure="false">Dane!$C$13</definedName>
     <definedName function="false" hidden="false" name="in_km_mon" vbProcedure="false">Dane!$C$15</definedName>
     <definedName function="false" hidden="false" name="in_km_pom" vbProcedure="false">Dane!$C$14</definedName>
-    <definedName function="false" hidden="false" name="in_konsA" vbProcedure="false">Dane!$C$60</definedName>
-    <definedName function="false" hidden="false" name="in_konsB" vbProcedure="false">Dane!$C$61</definedName>
+    <definedName function="false" hidden="false" name="in_konsA" vbProcedure="false">Dane!$C$61</definedName>
+    <definedName function="false" hidden="false" name="in_konsB" vbProcedure="false">Dane!$C$62</definedName>
     <definedName function="false" hidden="false" name="in_lok" vbProcedure="false">Dane!$C$12</definedName>
     <definedName function="false" hidden="false" name="in_magistrala" vbProcedure="false">Dane!$C$23</definedName>
     <definedName function="false" hidden="false" name="in_maskownice" vbProcedure="false">Dane!$C$25</definedName>
@@ -102,8 +103,8 @@
     <definedName function="false" hidden="false" name="in_NP" vbProcedure="false">Dane!$C$21</definedName>
     <definedName function="false" hidden="false" name="in_nr" vbProcedure="false">Dane!$C$8</definedName>
     <definedName function="false" hidden="false" name="in_opis" vbProcedure="false">Dane!$C$9</definedName>
-    <definedName function="false" hidden="false" name="in_osoby" vbProcedure="false">Dane!$C$51</definedName>
-    <definedName function="false" hidden="false" name="in_q2500" vbProcedure="false">Dane!$C$58</definedName>
+    <definedName function="false" hidden="false" name="in_osoby" vbProcedure="false">Dane!$C$52</definedName>
+    <definedName function="false" hidden="false" name="in_q2500" vbProcedure="false">Dane!$C$59</definedName>
     <definedName function="false" hidden="false" name="in_rozl_cena" vbProcedure="false">Dane!$C$49</definedName>
     <definedName function="false" hidden="false" name="in_rozl_dni" vbProcedure="false">Dane!$C$50</definedName>
     <definedName function="false" hidden="false" name="in_S" vbProcedure="false">Dane!$C$19</definedName>
@@ -115,10 +116,10 @@
     <definedName function="false" hidden="false" name="in_tir_cena" vbProcedure="false">Dane!$C$48</definedName>
     <definedName function="false" hidden="false" name="in_typ" vbProcedure="false">Dane!$C$18</definedName>
     <definedName function="false" hidden="false" name="in_utr_dod" vbProcedure="false">Dane!$C$26</definedName>
-    <definedName function="false" hidden="false" name="in_wyjazdy" vbProcedure="false">Dane!$C$52</definedName>
-    <definedName function="false" hidden="false" name="in_wzor" vbProcedure="false">Dane!$C$53</definedName>
-    <definedName function="false" hidden="false" name="in_zysk" vbProcedure="false">Dane!$C$56</definedName>
-    <definedName function="false" hidden="false" name="in_zysk2" vbProcedure="false">Dane!$C$57</definedName>
+    <definedName function="false" hidden="false" name="in_wyjazdy" vbProcedure="false">Dane!$C$53</definedName>
+    <definedName function="false" hidden="false" name="in_wzor" vbProcedure="false">Dane!$C$54</definedName>
+    <definedName function="false" hidden="false" name="in_zysk" vbProcedure="false">Dane!$C$57</definedName>
+    <definedName function="false" hidden="false" name="in_zysk2" vbProcedure="false">Dane!$C$58</definedName>
     <definedName function="false" hidden="false" name="m_barierki" vbProcedure="false">Obliczenia!$C$18</definedName>
     <definedName function="false" hidden="false" name="m_cena_D" vbProcedure="false">Obliczenia!$C$5</definedName>
     <definedName function="false" hidden="false" name="m_cena_NP" vbProcedure="false">Obliczenia!$C$7</definedName>
@@ -159,7 +160,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="360">
   <si>
     <t xml:space="preserve">KALKULATOR NK38 - DANE WEJŚCIOWE</t>
   </si>
@@ -336,6 +337,12 @@
   </si>
   <si>
     <t xml:space="preserve">puste = 0,5 dnia / TIR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nadpisz: koszt Spider Crane razem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">puste = cena za dzień x liczba dni</t>
   </si>
   <si>
     <t xml:space="preserve">Liczba osób na montażu</t>
@@ -1822,7 +1829,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:F70"/>
+  <dimension ref="B2:F71"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2322,9 +2329,7 @@
       <c r="B51" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="C51" s="10" t="n">
-        <v>4</v>
-      </c>
+      <c r="C51" s="13"/>
       <c r="E51" s="8" t="s">
         <v>60</v>
       </c>
@@ -2333,110 +2338,112 @@
       <c r="B52" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="C52" s="10"/>
+      <c r="C52" s="10" t="n">
+        <v>4</v>
+      </c>
       <c r="E52" s="8" t="s">
-        <v>16</v>
+        <v>62</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="C53" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="C53" s="10"/>
       <c r="E53" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="0" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="4" t="s">
+      <c r="C54" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="5"/>
+      <c r="E54" s="8" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="C56" s="14" t="n">
-        <v>0.14</v>
-      </c>
+      <c r="B56" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="0" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C57" s="14" t="n">
-        <v>0.1</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C58" s="14" t="n">
-        <f aca="false">c_q2500</f>
-        <v>0.07</v>
-      </c>
-      <c r="E58" s="8" t="s">
-        <v>69</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="C59" s="15" t="n">
-        <v>4.325</v>
+      <c r="C59" s="14" t="n">
+        <f aca="false">c_q2500</f>
+        <v>0.07</v>
+      </c>
+      <c r="E59" s="8" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="C60" s="13" t="n">
-        <v>40</v>
+        <v>72</v>
+      </c>
+      <c r="C60" s="15" t="n">
+        <v>4.325</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C61" s="13" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="0" t="s">
-        <v>73</v>
-      </c>
-      <c r="C62" s="6" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="4" t="s">
+      <c r="C62" s="13" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="C64" s="5"/>
-      <c r="D64" s="5"/>
-      <c r="E64" s="5"/>
+      <c r="C63" s="6" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B65" s="16" t="str">
-        <f aca="false">IF(OR(C39&lt;0,D39&lt;0),"BŁĄD: więcej zagłębień niż platform","ok")</f>
-        <v>ok</v>
-      </c>
-      <c r="C65" s="16"/>
-      <c r="D65" s="16"/>
-      <c r="E65" s="16"/>
+      <c r="B65" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C65" s="5"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="16" t="str">
-        <f aca="false">IF(OR(in_szer1_S+in_szer2_S&gt;in_S,in_szer1_D+in_szer2_D&gt;in_D),"BŁĄD: więcej szerokości niż platform","ok")</f>
+        <f aca="false">IF(OR(C39&lt;0,D39&lt;0),"BŁĄD: więcej zagłębień niż platform","ok")</f>
         <v>ok</v>
       </c>
       <c r="C66" s="16"/>
@@ -2445,7 +2452,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="16" t="str">
-        <f aca="false">IF(OR(in_dl500_S+in_dl540_S+in_dl550_S&gt;in_S,in_dl500_D+in_dl540_D+in_dl550_D&gt;in_D),"BŁĄD: więcej długości niż platform","ok")</f>
+        <f aca="false">IF(OR(in_szer1_S+in_szer2_S&gt;in_S,in_szer1_D+in_szer2_D&gt;in_D),"BŁĄD: więcej szerokości niż platform","ok")</f>
         <v>ok</v>
       </c>
       <c r="C67" s="16"/>
@@ -2454,7 +2461,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="16" t="str">
-        <f aca="false">IF(in_agregaty*6&lt;in_S+in_D+in_NP,"UWAGA: mniej niż 1 agregat na 6 platform","ok")</f>
+        <f aca="false">IF(OR(in_dl500_S+in_dl540_S+in_dl550_S&gt;in_S,in_dl500_D+in_dl540_D+in_dl550_D&gt;in_D),"BŁĄD: więcej długości niż platform","ok")</f>
         <v>ok</v>
       </c>
       <c r="C68" s="16"/>
@@ -2463,8 +2470,8 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="16" t="str">
-        <f aca="false">IF(in_S+in_D+in_NP=0,"UWAGA: brak platform",IF(in_tir=0,"UWAGA: brak transportów","ok"))</f>
-        <v>UWAGA: brak platform</v>
+        <f aca="false">IF(in_agregaty*6&lt;in_S+in_D+in_NP,"UWAGA: mniej niż 1 agregat na 6 platform","ok")</f>
+        <v>ok</v>
       </c>
       <c r="C69" s="16"/>
       <c r="D69" s="16"/>
@@ -2472,25 +2479,34 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="16" t="str">
-        <f aca="false">IF(AND(in_lok="Poza Krakowem",in_km=0),"UWAGA: brak odległości od Krakowa","ok")</f>
-        <v>UWAGA: brak odległości od Krakowa</v>
+        <f aca="false">IF(in_S+in_D+in_NP=0,"UWAGA: brak platform",IF(in_tir=0,"UWAGA: brak transportów","ok"))</f>
+        <v>UWAGA: brak platform</v>
       </c>
       <c r="C70" s="16"/>
       <c r="D70" s="16"/>
       <c r="E70" s="16"/>
     </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B71" s="16" t="str">
+        <f aca="false">IF(AND(in_lok="Poza Krakowem",in_km=0),"UWAGA: brak odległości od Krakowa","ok")</f>
+        <v>UWAGA: brak odległości od Krakowa</v>
+      </c>
+      <c r="C71" s="16"/>
+      <c r="D71" s="16"/>
+      <c r="E71" s="16"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B65:E65"/>
     <mergeCell ref="B66:E66"/>
     <mergeCell ref="B67:E67"/>
     <mergeCell ref="B68:E68"/>
     <mergeCell ref="B69:E69"/>
     <mergeCell ref="B70:E70"/>
+    <mergeCell ref="B71:E71"/>
   </mergeCells>
-  <conditionalFormatting sqref="B65:B70">
+  <conditionalFormatting sqref="B66:B71">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>B65&lt;&gt;"ok"</formula>
+      <formula>B66&lt;&gt;"ok"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
@@ -2502,11 +2518,11 @@
       <formula1>"NK38,NK37"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C53" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C54" type="list">
       <formula1>"Stary (poprawiony),Uproszczony"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C62" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C63" type="list">
       <formula1>"2000 kg,2500 kg,2000 kg + słupki,2500 kg + słupki"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2514,7 +2530,7 @@
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C51" type="whole">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C52" type="whole">
       <formula1>1</formula1>
       <formula2>12</formula2>
     </dataValidation>
@@ -2545,7 +2561,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2568,19 +2584,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2629,7 +2645,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C9" s="19" t="n">
         <f aca="false">Obliczenia!D73</f>
@@ -2650,7 +2666,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C10" s="19" t="n">
         <f aca="false">Obliczenia!D78</f>
@@ -2671,7 +2687,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C11" s="20" t="n">
         <f aca="false">Obliczenia!D74</f>
@@ -2692,7 +2708,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="0" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C12" s="19" t="n">
         <f aca="false">Obliczenia!D69</f>
@@ -2713,7 +2729,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C13" s="19" t="n">
         <f aca="false">Obliczenia!D76</f>
@@ -2734,7 +2750,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="0" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C14" s="19" t="n">
         <f aca="false">Obliczenia!D72</f>
@@ -2755,7 +2771,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="0" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C16" s="19" t="n">
         <f aca="false">Obliczenia!D54</f>
@@ -2776,7 +2792,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="0" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C17" s="19" t="n">
         <f aca="false">Obliczenia!D55</f>
@@ -2797,7 +2813,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="0" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C18" s="19" t="n">
         <f aca="false">Obliczenia!D58+Obliczenia!D59+Obliczenia!D60</f>
@@ -2818,7 +2834,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="0" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C19" s="19" t="n">
         <f aca="false">Obliczenia!D63+Obliczenia!D61+Obliczenia!D62</f>
@@ -2839,7 +2855,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="0" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C20" s="19" t="n">
         <f aca="false">Obliczenia!D57+Obliczenia!D64+Obliczenia!D56</f>
@@ -2860,7 +2876,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="0" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C21" s="19" t="n">
         <f aca="false">Obliczenia!D67+Obliczenia!D68+Obliczenia!D70</f>
@@ -2881,7 +2897,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="11" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C23" s="21" t="n">
         <f aca="false">Obliczenia!D51</f>
@@ -2902,7 +2918,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C24" s="21" t="n">
         <f aca="false">Obliczenia!D52</f>
@@ -2923,7 +2939,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="0" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C25" s="22" t="n">
         <f aca="false">Obliczenia!D50</f>
@@ -2944,18 +2960,18 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="0" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C28" s="19" t="n">
         <f aca="false">Obliczenia!F71-Obliczenia!D71</f>
@@ -2968,7 +2984,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="0" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C29" s="19" t="n">
         <f aca="false">Obliczenia!F71-Obliczenia!D71+(c_slupek22-c_slupek)*m_MP*e_mnoznik</f>
@@ -2981,7 +2997,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="0" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C30" s="19" t="n">
         <f aca="false">m_malowanie*e_mnoznik</f>
@@ -3000,30 +3016,30 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F33" s="17" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G33" s="17" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H33" s="17" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C34" s="19" t="n">
         <f aca="false">Obliczenia!I71</f>
@@ -3052,7 +3068,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C35" s="19" t="n">
         <f aca="false">Obliczenia!I73</f>
@@ -3081,7 +3097,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="0" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C36" s="23" t="n">
         <f aca="false">Obliczenia!I51</f>
@@ -3110,7 +3126,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C37" s="23" t="n">
         <f aca="false">Obliczenia!I48</f>
@@ -3139,7 +3155,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C38" s="19" t="n">
         <f aca="false">Obliczenia!I57+Obliczenia!I64</f>
@@ -3168,12 +3184,12 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
@@ -3182,7 +3198,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C42" s="16" t="str">
         <f aca="false">in_typ&amp;": "&amp;IF(in_S&gt;0,in_S&amp;" x S (2 MP)  ","")&amp;IF(in_D&gt;0,in_D&amp;" x D (4 MP)  ","")&amp;IF(in_NP&gt;0,in_NP&amp;" x N.P.  ","")&amp;"= "&amp;m_MP&amp;" MP"</f>
@@ -3210,7 +3226,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C44" s="16" t="str">
         <f aca="false">IF(t_zaglebienia="","standard 170 cm",t_zaglebienia)</f>
@@ -3224,7 +3240,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C45" s="16" t="str">
         <f aca="false">IF(t_wymiary="","standard",t_wymiary)</f>
@@ -3238,7 +3254,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C46" s="16" t="str">
         <f aca="false">in_magistrala&amp;" x 6 m  /  "&amp;in_barierki&amp;" szt.  /  "&amp;in_maskownice&amp;" szt."</f>
@@ -3252,7 +3268,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C47" s="16" t="str">
         <f aca="false">m_utr&amp;" (z magistrali i barierek "&amp;m_utr_auto&amp;", ręcznie "&amp;in_utr_dod&amp;")"</f>
@@ -3280,7 +3296,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C49" s="16" t="str">
         <f aca="false">e_km_pom&amp;" / "&amp;e_km_mon&amp;" km"</f>
@@ -3294,7 +3310,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C50" s="16" t="str">
         <f aca="false">in_tir&amp;" TIR x "&amp;TEXT(in_tir_cena,"#,##0")&amp;" zł, rozładunek sprzętu "&amp;TEXT(in_rozl_cena,"#,##0")&amp;" zł jednorazowo, "&amp;e_rozl_dni&amp;" dni"</f>
@@ -3308,7 +3324,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="0" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C51" s="16" t="str">
         <f aca="false">in_osoby&amp;" osób, średnia stawka "&amp;TEXT(Obliczenia!D41,"#,##0")&amp;" zł/dzień"</f>
@@ -3322,7 +3338,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="0" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C52" s="16" t="str">
         <f aca="false">e_dzw_dni&amp;" dni"</f>
@@ -3336,7 +3352,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C53" s="16" t="str">
         <f aca="false">Obliczenia!D51&amp;" dni pracy = "&amp;Obliczenia!D48&amp;IF(e_krk," dni"," tyg.")&amp;", "&amp;TEXT(Obliczenia!D50,"0.0")&amp;" osobodni"</f>
@@ -3350,7 +3366,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C54" s="16" t="str">
         <f aca="false">Obliczenia!F51&amp;" dni pracy = "&amp;Obliczenia!F48&amp;IF(e_krk," dni"," tyg.")&amp;", "&amp;TEXT(Obliczenia!F50,"0.0")&amp;" osobodni"</f>
@@ -3364,7 +3380,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C55" s="16" t="str">
         <f aca="false">TEXT(in_zysk,"0.0%")&amp;" / "&amp;TEXT(in_zysk2,"0.0%")</f>
@@ -3378,7 +3394,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C56" s="16" t="str">
         <f aca="false">TEXT(in_q2500,"0.0%")</f>
@@ -3392,7 +3408,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="0" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C57" s="16" t="str">
         <f aca="false">in_wzor</f>
@@ -3406,7 +3422,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C58" s="16" t="str">
         <f aca="false">TEXT(in_konsA*m_MP*12,"#,##0")&amp;" / "&amp;TEXT(in_konsB*m_MP*12,"#,##0")&amp;" zł  (przegląd półroczny "&amp;TEXT(in_konsA*m_MP*6,"#,##0")&amp;" / "&amp;TEXT(in_konsB*m_MP*6,"#,##0")&amp;" zł)"</f>
@@ -3420,7 +3436,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C59" s="16" t="str">
         <f aca="false">in_opis&amp;""</f>
@@ -3434,16 +3450,16 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="11" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C61" s="0" t="str">
-        <f aca="false">IF(COUNTIF(Dane!B65:B70,"ok")=6,"wszystko ok","sprawdź arkusz Dane")</f>
+        <f aca="false">IF(COUNTIF(Dane!B66:B71,"ok")=6,"wszystko ok","sprawdź arkusz Dane")</f>
         <v>sprawdź arkusz Dane</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C63" s="5"/>
       <c r="D63" s="5"/>
@@ -3454,7 +3470,7 @@
     </row>
     <row r="64" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="24" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C64" s="24"/>
       <c r="D64" s="24"/>
@@ -3465,7 +3481,7 @@
     </row>
     <row r="65" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="24" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C65" s="24"/>
       <c r="D65" s="24"/>
@@ -3476,7 +3492,7 @@
     </row>
     <row r="66" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B66" s="24" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C66" s="24"/>
       <c r="D66" s="24"/>
@@ -3487,7 +3503,7 @@
     </row>
     <row r="67" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="24" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C67" s="24"/>
       <c r="D67" s="24"/>
@@ -3498,7 +3514,7 @@
     </row>
     <row r="68" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="24" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C68" s="24"/>
       <c r="D68" s="24"/>
@@ -3509,7 +3525,7 @@
     </row>
     <row r="69" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B69" s="24" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C69" s="24"/>
       <c r="D69" s="24"/>
@@ -3582,7 +3598,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -3591,12 +3607,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -3604,90 +3620,90 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>32500</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="0" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>700</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>0.61</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C9" s="14" t="n">
         <v>0.85</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1170</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1560</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1820</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>3110</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3698,34 +3714,34 @@
         <v>2340</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C15" s="25" t="n">
         <v>0.00127</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C16" s="14" t="n">
         <v>0.07</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="4" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
@@ -3733,107 +3749,107 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="0" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>6500</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="0" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1500</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="0" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>200</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>500</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>50</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="0" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1080</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="0" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1175</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="0" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1250</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="0" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C26" s="26" t="n">
         <f aca="false">0.2*11+0.4*11+2*14+6*11+6*5+6*10</f>
         <v>190.6</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -3841,51 +3857,51 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="0" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>600</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="0" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>700</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="0" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1000</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="0" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1800</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="4" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
@@ -3893,73 +3909,73 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="0" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>6400</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>13500</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="0" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>200</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="0" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1700</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="0" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>6300</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="0" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C38" s="9" t="n">
         <v>0.37</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="4" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
@@ -3967,117 +3983,117 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="0" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C40" s="9" t="n">
         <v>5.5</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="0" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C41" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="0" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C42" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="0" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C43" s="9" t="n">
         <v>0.5</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="0" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C44" s="9" t="n">
         <v>0.5</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="0" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C45" s="9" t="n">
         <v>0.5</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="0" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>2400</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="0" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C47" s="9" t="n">
         <v>5</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="0" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C48" s="9" t="n">
         <v>0.6</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="0" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C49" s="9" t="n">
         <v>5</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="4" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5"/>
@@ -4085,84 +4101,84 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="0" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C51" s="9" t="n">
         <v>50</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="0" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C52" s="9" t="n">
         <v>20</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="0" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C53" s="9" t="n">
         <v>650</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="0" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C54" s="9" t="n">
         <v>12</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="0" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C55" s="26" t="n">
         <v>9.4</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="0" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C56" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="0" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C57" s="9" t="n">
         <v>2</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5"/>
@@ -4170,62 +4186,62 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="0" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>500</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="0" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>400</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="0" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C61" s="13" t="n">
         <v>350</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="0" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C62" s="13" t="n">
         <v>45</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="0" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C63" s="13" t="n">
         <v>130</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="4" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C64" s="5"/>
       <c r="D64" s="5"/>
@@ -4233,40 +4249,40 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="0" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C65" s="14" t="n">
         <v>0.005</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="0" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C66" s="14" t="n">
         <v>0.025</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="0" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C67" s="14" t="n">
         <v>0.14</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="4" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C69" s="5"/>
       <c r="D69" s="5"/>
@@ -4274,13 +4290,13 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="11" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4384,7 +4400,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="4" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C81" s="5"/>
       <c r="D81" s="5"/>
@@ -4393,24 +4409,24 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="11" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C82" s="11" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D82" s="11" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E82" s="11" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="F82" s="11" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="0" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C83" s="29" t="n">
         <v>45</v>
@@ -4422,12 +4438,12 @@
         <v>9.6</v>
       </c>
       <c r="F83" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="0" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C84" s="29" t="n">
         <v>8</v>
@@ -4439,12 +4455,12 @@
         <v>4</v>
       </c>
       <c r="F84" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="0" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C85" s="29" t="n">
         <v>36</v>
@@ -4456,12 +4472,12 @@
         <v>2</v>
       </c>
       <c r="F85" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="0" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C86" s="29" t="n">
         <v>90</v>
@@ -4473,12 +4489,12 @@
         <v>2</v>
       </c>
       <c r="F86" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="0" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C87" s="29" t="n">
         <v>207.28</v>
@@ -4490,12 +4506,12 @@
         <v>2</v>
       </c>
       <c r="F87" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="0" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C88" s="29" t="n">
         <v>40.14</v>
@@ -4507,12 +4523,12 @@
         <v>2</v>
       </c>
       <c r="F88" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="0" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C89" s="29" t="n">
         <v>3.3</v>
@@ -4524,12 +4540,12 @@
         <v>2</v>
       </c>
       <c r="F89" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="0" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C90" s="29" t="n">
         <v>10.8</v>
@@ -4541,12 +4557,12 @@
         <v>2</v>
       </c>
       <c r="F90" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="0" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C91" s="29" t="n">
         <v>10.95</v>
@@ -4558,12 +4574,12 @@
         <v>2</v>
       </c>
       <c r="F91" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="0" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C92" s="29" t="n">
         <v>3.81</v>
@@ -4575,12 +4591,12 @@
         <v>2</v>
       </c>
       <c r="F92" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="0" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C93" s="29" t="n">
         <v>2.84</v>
@@ -4592,12 +4608,12 @@
         <v>4</v>
       </c>
       <c r="F93" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="0" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C94" s="29" t="n">
         <v>4.4</v>
@@ -4609,12 +4625,12 @@
         <v>4</v>
       </c>
       <c r="F94" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="0" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C95" s="29" t="n">
         <f aca="false">2*25.71+2*22.85</f>
@@ -4627,12 +4643,12 @@
         <v>1</v>
       </c>
       <c r="F95" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="0" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C96" s="29" t="n">
         <v>345</v>
@@ -4644,12 +4660,12 @@
         <v>0</v>
       </c>
       <c r="F96" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="0" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C97" s="29" t="n">
         <v>546</v>
@@ -4661,12 +4677,12 @@
         <v>1</v>
       </c>
       <c r="F97" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="0" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C98" s="29" t="n">
         <v>2.98</v>
@@ -4678,12 +4694,12 @@
         <v>208</v>
       </c>
       <c r="F98" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="0" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C99" s="29" t="n">
         <f aca="false">3.09+4.99</f>
@@ -4696,12 +4712,12 @@
         <v>20</v>
       </c>
       <c r="F99" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B100" s="0" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C100" s="29" t="n">
         <v>5.4</v>
@@ -4713,12 +4729,12 @@
         <v>1</v>
       </c>
       <c r="F100" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B101" s="0" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C101" s="29" t="n">
         <v>300</v>
@@ -4730,12 +4746,12 @@
         <v>1</v>
       </c>
       <c r="F101" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B102" s="0" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C102" s="29" t="n">
         <v>40</v>
@@ -4747,12 +4763,12 @@
         <v>1</v>
       </c>
       <c r="F102" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B103" s="0" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C103" s="29" t="n">
         <v>172</v>
@@ -4764,12 +4780,12 @@
         <v>0</v>
       </c>
       <c r="F103" s="30" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B104" s="0" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C104" s="29" t="n">
         <v>207</v>
@@ -4781,12 +4797,12 @@
         <v>1</v>
       </c>
       <c r="F104" s="30" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="0" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C105" s="29" t="n">
         <f aca="false">120+55+65</f>
@@ -4799,12 +4815,12 @@
         <v>1</v>
       </c>
       <c r="F105" s="30" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B106" s="0" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C106" s="29" t="n">
         <f aca="false">50+40</f>
@@ -4817,12 +4833,12 @@
         <v>1</v>
       </c>
       <c r="F106" s="30" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B107" s="0" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C107" s="29" t="n">
         <f aca="false">14+9+25+5+9+30</f>
@@ -4835,12 +4851,12 @@
         <v>0</v>
       </c>
       <c r="F107" s="30" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B108" s="0" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C108" s="29" t="n">
         <f aca="false">14+18+25+7+18+30</f>
@@ -4853,12 +4869,12 @@
         <v>1</v>
       </c>
       <c r="F108" s="30" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="0" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C109" s="29" t="n">
         <f aca="false">70+14+34+32+20</f>
@@ -4871,7 +4887,7 @@
         <v>1</v>
       </c>
       <c r="F109" s="30" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>
@@ -4902,7 +4918,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -4919,13 +4935,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="0" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C5" s="31" t="n">
         <f aca="false">c_cena_D+IF(in_typ="NK37",c_doplata_NK37,0)</f>
@@ -4934,7 +4950,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="0" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C6" s="31" t="n">
         <f aca="false">c_wsp_S*m_cena_D</f>
@@ -4943,7 +4959,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="0" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C7" s="31" t="n">
         <f aca="false">c_wsp_NP*m_cena_D</f>
@@ -4952,7 +4968,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="0" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C8" s="32" t="n">
         <f aca="false">in_D+in_NP</f>
@@ -4961,7 +4977,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="0" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C9" s="32" t="n">
         <f aca="false">in_S+in_D+in_NP</f>
@@ -4970,7 +4986,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="0" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C10" s="32" t="n">
         <f aca="false">2*in_S+2*in_NP+4*in_D</f>
@@ -4979,7 +4995,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="0" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C11" s="31" t="n">
         <f aca="false">m_cena_S*in_S+c_szer_260*in_szer1_S+c_szer_270*in_szer2_S+SUMPRODUCT(in_gl_S,t_gl_doplata)+c_dl_500*in_dl500_S+CEILING(m_cena_S*c_dl_wsp*10,100)*in_dl540_S+CEILING(m_cena_S*c_dl_wsp*20,100)*in_dl550_S</f>
@@ -4988,7 +5004,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="0" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C12" s="31" t="n">
         <f aca="false">m_cena_D*in_D+c_szer_520*in_szer1_D+c_szer_540*in_szer2_D+SUMPRODUCT(in_gl_D,t_gl_doplata)+c_dl_500*in_dl500_D+m_cena_D*c_dl_wsp*10*in_dl540_D+m_cena_D*c_dl_wsp*20*in_dl550_D</f>
@@ -4997,7 +5013,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="0" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C13" s="31" t="n">
         <f aca="false">m_cena_NP*in_NP</f>
@@ -5006,7 +5022,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="0" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C14" s="32" t="n">
         <f aca="false">SUMPRODUCT((t_gl_silownik=2000)*(in_gl_S+in_gl_D))</f>
@@ -5015,7 +5031,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="0" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C15" s="32" t="n">
         <f aca="false">SUMPRODUCT((t_gl_silownik=2250)*(in_gl_S+in_gl_D))</f>
@@ -5024,7 +5040,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="0" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C16" s="32" t="n">
         <f aca="false">m_platformy-m_sil_2000-m_sil_2250</f>
@@ -5033,7 +5049,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C17" s="31" t="n">
         <f aca="false">in_agregaty*(c_agregat+c_hydr_drobne+c_olej+c_transp_agregatu)+m_platformy*c_transp_silownikow+2*(c_sil_1700*m_sil_std+c_sil_2000*m_sil_2000+c_sil_2250*m_sil_2250)+in_magistrala*c_magistrala+SUMPRODUCT((t_sk_grupa="Hydraulika")*t_sk_cena*(t_sk_S*in_S+t_sk_D*m_DN))</f>
@@ -5042,7 +5058,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="0" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C18" s="31" t="n">
         <f aca="false">in_barierki*c_barierka+in_maskownice*c_maskownica</f>
@@ -5051,7 +5067,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="0" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C19" s="31" t="n">
         <f aca="false">in_agregaty*c_skrzynka_zasil+SUMPRODUCT((t_sk_grupa="Elektryka")*t_sk_cena*(t_sk_S*in_S+t_sk_D*m_DN))</f>
@@ -5060,7 +5076,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="0" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="C20" s="31" t="n">
         <f aca="false">in_agregaty*c_admin+SUMPRODUCT((t_sk_grupa="Mechanika")*t_sk_cena*(t_sk_S*in_S+t_sk_D*m_DN))</f>
@@ -5069,7 +5085,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="11" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C21" s="33" t="n">
         <f aca="false">m_plat_S+m_plat_D+m_plat_NP+m_hydraulika+m_barierki+m_elektryka+m_mechanika</f>
@@ -5078,7 +5094,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="11" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C22" s="33" t="n">
         <f aca="false">m_suma_2000*(1+in_q2500)</f>
@@ -5087,7 +5103,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="0" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C23" s="31" t="n">
         <f aca="false">c_mal_S*in_S+c_mal_D*m_DN+c_mal_bar*in_barierki</f>
@@ -5096,7 +5112,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="0" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C24" s="34" t="n">
         <f aca="false">ROUNDUP(in_magistrala*c_osd_magistrala+(in_barierki+in_maskownice)*c_osd_barierka,0)</f>
@@ -5105,7 +5121,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="0" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C25" s="34" t="n">
         <f aca="false">m_utr_auto+in_utr_dod</f>
@@ -5114,13 +5130,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="0" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C28" s="35" t="b">
         <f aca="false">in_lok="Kraków"</f>
@@ -5129,7 +5145,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="0" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C29" s="34" t="n">
         <f aca="false">IF(ISBLANK(in_km_pom),IF(e_krk,c_km_krakow,in_km),in_km_pom)</f>
@@ -5138,7 +5154,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="0" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C30" s="34" t="n">
         <f aca="false">IF(ISBLANK(in_km_mon),IF(e_krk,c_km_krakow,in_km+c_km_dodatek),in_km_mon)</f>
@@ -5147,7 +5163,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="0" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C31" s="34" t="n">
         <f aca="false">IF(ISBLANK(in_rozl_dni),c_rozl_TIR*in_tir,in_rozl_dni)</f>
@@ -5156,7 +5172,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="0" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C32" s="34" t="n">
         <f aca="false">(c_pomiary_osoby+c_odbiory_osoby)*IF(in_wzor="Uproszczony",2*e_km_pom/c_km_dzien*1,(1+0.1*MAX(0,800-e_km_pom)/100)*e_km_pom*1/500)</f>
@@ -5165,7 +5181,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="0" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C33" s="32" t="n">
         <f aca="false">ROUNDUP(m_DN/c_dzwig_D+in_S*c_dzwig_wspS/c_dzwig_D,0)</f>
@@ -5174,7 +5190,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C34" s="36" t="n">
         <f aca="false">(1+c_podatek*(c_gdw+in_zysk))/(1-(c_kob+c_gdw+in_zysk))</f>
@@ -5183,7 +5199,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="4" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
@@ -5192,7 +5208,7 @@
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
       <c r="I36" s="4" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="J36" s="5"/>
       <c r="K36" s="5"/>
@@ -5202,42 +5218,42 @@
     </row>
     <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="11" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="D37" s="37" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E37" s="37" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F37" s="37" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G37" s="37" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I37" s="37" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J37" s="37" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K37" s="37" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="L37" s="37" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="M37" s="37" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="N37" s="37" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="0" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="D38" s="32" t="n">
         <v>0</v>
@@ -5278,7 +5294,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="0" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="D39" s="32" t="n">
         <v>0</v>
@@ -5319,7 +5335,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="0" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D40" s="32" t="n">
         <f aca="false">in_osoby</f>
@@ -5358,7 +5374,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="0" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D41" s="31" t="n">
         <f aca="false">(c_stawka_1+IF(D40&gt;=2,c_stawka_2,0)+MAX(0,D40-2)*c_stawka_n)/D40</f>
@@ -5403,7 +5419,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="0" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="D42" s="34" t="n">
         <f aca="false">c_osd_S*in_S+c_osd_D*in_D+c_osd_NP*in_NP+m_utr+D39*c_slupek_rbd*m_MP</f>
@@ -5448,7 +5464,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="0" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D43" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*1,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*1/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*1,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*1/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5493,7 +5509,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="0" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D44" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D43,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D43/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D43,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D43/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5538,7 +5554,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="0" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="D45" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D44,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D44/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D44,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D44/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5583,7 +5599,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="0" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D46" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D45,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D45/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D45,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D45/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5628,7 +5644,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="0" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="D47" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D46,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D46/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D46,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D46/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5673,7 +5689,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="11" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D48" s="38" t="n">
         <f aca="false">IF(ISBLANK(in_wyjazdy),D47,in_wyjazdy)</f>
@@ -5718,7 +5734,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="0" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="D49" s="34" t="n">
         <f aca="false">(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D48,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D48/500)))</f>
@@ -5763,7 +5779,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="0" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D50" s="34" t="n">
         <f aca="false">D42+D49</f>
@@ -5808,7 +5824,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="11" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D51" s="38" t="n">
         <f aca="false">CEILING(D50/D40,1)</f>
@@ -5853,7 +5869,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="11" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="D52" s="38" t="n">
         <f aca="false">IF(e_krk,CEILING(D51/c_dni_tydzien,1),D48)</f>
@@ -5898,7 +5914,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="0" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D53" s="34" t="n">
         <f aca="false">2*(e_km_mon*D48+2*e_km_pom)</f>
@@ -5943,7 +5959,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="0" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D54" s="31" t="n">
         <f aca="false">IF(D38=1,m_suma_2500,m_suma_2000)</f>
@@ -5988,7 +6004,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="0" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D55" s="31" t="n">
         <f aca="false">D39*c_slupek*m_MP</f>
@@ -6033,7 +6049,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="0" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D56" s="31" t="n">
         <f aca="false">D53/100*ROUNDUP(c_spalanie*c_paliwo,0)</f>
@@ -6078,7 +6094,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="0" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D57" s="31" t="n">
         <f aca="false">IF(e_krk,0,c_hotel*(D51+1)*D40)</f>
@@ -6123,7 +6139,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="0" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D58" s="31" t="n">
         <f aca="false">in_tir_cena*in_tir</f>
@@ -6168,52 +6184,52 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="0" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="D59" s="31" t="n">
-        <f aca="false">c_dzwig*e_dzw_dni</f>
+        <f aca="false">IF(ISBLANK(in_dzwig_koszt),c_dzwig*e_dzw_dni,in_dzwig_koszt)</f>
         <v>0</v>
       </c>
       <c r="E59" s="31" t="n">
-        <f aca="false">c_dzwig*e_dzw_dni</f>
+        <f aca="false">IF(ISBLANK(in_dzwig_koszt),c_dzwig*e_dzw_dni,in_dzwig_koszt)</f>
         <v>0</v>
       </c>
       <c r="F59" s="31" t="n">
-        <f aca="false">c_dzwig*e_dzw_dni</f>
+        <f aca="false">IF(ISBLANK(in_dzwig_koszt),c_dzwig*e_dzw_dni,in_dzwig_koszt)</f>
         <v>0</v>
       </c>
       <c r="G59" s="31" t="n">
-        <f aca="false">c_dzwig*e_dzw_dni</f>
+        <f aca="false">IF(ISBLANK(in_dzwig_koszt),c_dzwig*e_dzw_dni,in_dzwig_koszt)</f>
         <v>0</v>
       </c>
       <c r="I59" s="31" t="n">
-        <f aca="false">c_dzwig*e_dzw_dni</f>
+        <f aca="false">IF(ISBLANK(in_dzwig_koszt),c_dzwig*e_dzw_dni,in_dzwig_koszt)</f>
         <v>0</v>
       </c>
       <c r="J59" s="31" t="n">
-        <f aca="false">c_dzwig*e_dzw_dni</f>
+        <f aca="false">IF(ISBLANK(in_dzwig_koszt),c_dzwig*e_dzw_dni,in_dzwig_koszt)</f>
         <v>0</v>
       </c>
       <c r="K59" s="31" t="n">
-        <f aca="false">c_dzwig*e_dzw_dni</f>
+        <f aca="false">IF(ISBLANK(in_dzwig_koszt),c_dzwig*e_dzw_dni,in_dzwig_koszt)</f>
         <v>0</v>
       </c>
       <c r="L59" s="31" t="n">
-        <f aca="false">c_dzwig*e_dzw_dni</f>
+        <f aca="false">IF(ISBLANK(in_dzwig_koszt),c_dzwig*e_dzw_dni,in_dzwig_koszt)</f>
         <v>0</v>
       </c>
       <c r="M59" s="31" t="n">
-        <f aca="false">c_dzwig*e_dzw_dni</f>
+        <f aca="false">IF(ISBLANK(in_dzwig_koszt),c_dzwig*e_dzw_dni,in_dzwig_koszt)</f>
         <v>0</v>
       </c>
       <c r="N59" s="31" t="n">
-        <f aca="false">c_dzwig*e_dzw_dni</f>
+        <f aca="false">IF(ISBLANK(in_dzwig_koszt),c_dzwig*e_dzw_dni,in_dzwig_koszt)</f>
         <v>0</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="0" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="D60" s="31" t="n">
         <f aca="false">in_rozl_cena</f>
@@ -6258,7 +6274,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="0" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D61" s="31" t="n">
         <f aca="false">D41*e_rozl_dni*D40</f>
@@ -6303,7 +6319,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="0" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="D62" s="31" t="n">
         <f aca="false">D41*(D49-D40*e_rozl_dni)</f>
@@ -6348,7 +6364,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="0" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D63" s="31" t="n">
         <f aca="false">IF(D48&gt;0,D41*D42,0)</f>
@@ -6393,7 +6409,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="0" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="D64" s="31" t="n">
         <f aca="false">IF(e_krk,0,c_dieta*D50)</f>
@@ -6438,7 +6454,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="11" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="D65" s="33" t="n">
         <f aca="false">SUM(D54:D64)</f>
@@ -6483,7 +6499,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="0" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="D66" s="31" t="n">
         <f aca="false">D65/(1-(c_kob+c_gdw+in_zysk))</f>
@@ -6528,7 +6544,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="0" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="D67" s="31" t="n">
         <f aca="false">D66*c_kob</f>
@@ -6573,7 +6589,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="0" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D68" s="31" t="n">
         <f aca="false">D66*c_gdw</f>
@@ -6618,7 +6634,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="0" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D69" s="31" t="n">
         <f aca="false">D66*in_zysk</f>
@@ -6663,7 +6679,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="0" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D70" s="31" t="n">
         <f aca="false">c_podatek*(D61+D62+D63+D64+D68+D69)</f>
@@ -6708,7 +6724,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="11" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D71" s="33" t="n">
         <f aca="false">D66+D70</f>
@@ -6753,7 +6769,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="0" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="D72" s="31" t="n">
         <f aca="false">D71-D69</f>
@@ -6798,7 +6814,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D73" s="31" t="n">
         <f aca="false">IF(m_MP&gt;0,D71/m_MP,0)</f>
@@ -6843,7 +6859,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="0" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D74" s="39" t="n">
         <f aca="false">D73/in_eur</f>
@@ -6888,7 +6904,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="0" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="D75" s="31" t="n">
         <f aca="false">D65/(1-(c_kob+c_gdw+in_zysk2))</f>
@@ -6933,7 +6949,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="0" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="D76" s="31" t="n">
         <f aca="false">D75*in_zysk2</f>
@@ -6978,7 +6994,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="11" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="D77" s="33" t="n">
         <f aca="false">D75+c_podatek*(D61+D62+D63+D64+D75*(c_gdw+in_zysk2))</f>
@@ -7023,7 +7039,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D78" s="31" t="n">
         <f aca="false">IF(m_MP&gt;0,D77/m_MP,0)</f>

</xml_diff>

<commit_message>
Kalkulator: zysk z narzutem jak w Excelu, zapis wycen z nadpisywaniem, poprawki
- zysk z narzutem = cena - koszt rzeczywisty (zysk + GDW), koszt rzeczywisty = koszty + KOB + podatek (jak J43/J44); silnik, model, Excel, raport, panel
- wymiary niestandardowe nie znikają po powrocie z pulpitu ani po wczytaniu wyceny
- zapis wyceny: nadpisz wczytaną albo zapisz jako nową z nazwą z datą; usuwanie wycen z pulpitu
- potwierdzenia usuwania w miejscu przycisku, bez przerysowania ekranu
- edytor szablonu: przycisk Zapisz szablon i informacja o zapisie; pole tonażu w jednej linii

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/Kalkulator_NK38_v1.xlsx
+++ b/kalkulator-nk38/Kalkulator_NK38_v1.xlsx
@@ -160,7 +160,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="362">
   <si>
     <t xml:space="preserve">KALKULATOR NK38 - DANE WEJŚCIOWE</t>
   </si>
@@ -420,6 +420,9 @@
     <t xml:space="preserve">Cena za MP [EUR] - zysk A</t>
   </si>
   <si>
+    <t xml:space="preserve">Zysk z narzutem A [zł]</t>
+  </si>
+  <si>
     <t xml:space="preserve">Zysk A [zł]</t>
   </si>
   <si>
@@ -1228,6 +1231,9 @@
   </si>
   <si>
     <t xml:space="preserve">Koszt rzeczywisty (dawne K43)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zysk z narzutem (dawne J44 = zysk + GDW)</t>
   </si>
   <si>
     <t xml:space="preserve">Cena za MP [EUR]</t>
@@ -2550,7 +2556,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:H69"/>
+  <dimension ref="B2:H70"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2627,19 +2633,19 @@
         <v>CENA NETTO - ZYSK B 10.0%</v>
       </c>
       <c r="C8" s="18" t="n">
-        <f aca="false">Obliczenia!D77</f>
+        <f aca="false">Obliczenia!D78</f>
         <v>1756.40166666667</v>
       </c>
       <c r="D8" s="18" t="n">
-        <f aca="false">Obliczenia!E77</f>
+        <f aca="false">Obliczenia!E78</f>
         <v>1756.40166666667</v>
       </c>
       <c r="E8" s="18" t="n">
-        <f aca="false">Obliczenia!F77</f>
+        <f aca="false">Obliczenia!F78</f>
         <v>1756.40166666667</v>
       </c>
       <c r="F8" s="18" t="n">
-        <f aca="false">Obliczenia!G77</f>
+        <f aca="false">Obliczenia!G78</f>
         <v>1756.40166666667</v>
       </c>
     </row>
@@ -2648,19 +2654,19 @@
         <v>83</v>
       </c>
       <c r="C9" s="19" t="n">
-        <f aca="false">Obliczenia!D73</f>
+        <f aca="false">Obliczenia!D74</f>
         <v>0</v>
       </c>
       <c r="D9" s="19" t="n">
-        <f aca="false">Obliczenia!E73</f>
+        <f aca="false">Obliczenia!E74</f>
         <v>0</v>
       </c>
       <c r="E9" s="19" t="n">
-        <f aca="false">Obliczenia!F73</f>
+        <f aca="false">Obliczenia!F74</f>
         <v>0</v>
       </c>
       <c r="F9" s="19" t="n">
-        <f aca="false">Obliczenia!G73</f>
+        <f aca="false">Obliczenia!G74</f>
         <v>0</v>
       </c>
     </row>
@@ -2669,19 +2675,19 @@
         <v>84</v>
       </c>
       <c r="C10" s="19" t="n">
-        <f aca="false">Obliczenia!D78</f>
+        <f aca="false">Obliczenia!D79</f>
         <v>0</v>
       </c>
       <c r="D10" s="19" t="n">
-        <f aca="false">Obliczenia!E78</f>
+        <f aca="false">Obliczenia!E79</f>
         <v>0</v>
       </c>
       <c r="E10" s="19" t="n">
-        <f aca="false">Obliczenia!F78</f>
+        <f aca="false">Obliczenia!F79</f>
         <v>0</v>
       </c>
       <c r="F10" s="19" t="n">
-        <f aca="false">Obliczenia!G78</f>
+        <f aca="false">Obliczenia!G79</f>
         <v>0</v>
       </c>
     </row>
@@ -2690,19 +2696,19 @@
         <v>85</v>
       </c>
       <c r="C11" s="20" t="n">
-        <f aca="false">Obliczenia!D74</f>
+        <f aca="false">Obliczenia!D75</f>
         <v>0</v>
       </c>
       <c r="D11" s="20" t="n">
-        <f aca="false">Obliczenia!E74</f>
+        <f aca="false">Obliczenia!E75</f>
         <v>0</v>
       </c>
       <c r="E11" s="20" t="n">
-        <f aca="false">Obliczenia!F74</f>
+        <f aca="false">Obliczenia!F75</f>
         <v>0</v>
       </c>
       <c r="F11" s="20" t="n">
-        <f aca="false">Obliczenia!G74</f>
+        <f aca="false">Obliczenia!G75</f>
         <v>0</v>
       </c>
     </row>
@@ -2711,20 +2717,20 @@
         <v>86</v>
       </c>
       <c r="C12" s="19" t="n">
-        <f aca="false">Obliczenia!D69</f>
-        <v>247.024096385542</v>
+        <f aca="false">Obliczenia!D73</f>
+        <v>291.135542168675</v>
       </c>
       <c r="D12" s="19" t="n">
-        <f aca="false">Obliczenia!E69</f>
-        <v>247.024096385542</v>
+        <f aca="false">Obliczenia!E73</f>
+        <v>291.135542168675</v>
       </c>
       <c r="E12" s="19" t="n">
-        <f aca="false">Obliczenia!F69</f>
-        <v>247.024096385542</v>
+        <f aca="false">Obliczenia!F73</f>
+        <v>291.135542168675</v>
       </c>
       <c r="F12" s="19" t="n">
-        <f aca="false">Obliczenia!G69</f>
-        <v>247.024096385542</v>
+        <f aca="false">Obliczenia!G73</f>
+        <v>291.135542168675</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2732,20 +2738,20 @@
         <v>87</v>
       </c>
       <c r="C13" s="19" t="n">
-        <f aca="false">Obliczenia!D76</f>
-        <v>168.333333333333</v>
+        <f aca="false">Obliczenia!D69</f>
+        <v>247.024096385542</v>
       </c>
       <c r="D13" s="19" t="n">
-        <f aca="false">Obliczenia!E76</f>
-        <v>168.333333333333</v>
+        <f aca="false">Obliczenia!E69</f>
+        <v>247.024096385542</v>
       </c>
       <c r="E13" s="19" t="n">
-        <f aca="false">Obliczenia!F76</f>
-        <v>168.333333333333</v>
+        <f aca="false">Obliczenia!F69</f>
+        <v>247.024096385542</v>
       </c>
       <c r="F13" s="19" t="n">
-        <f aca="false">Obliczenia!G76</f>
-        <v>168.333333333333</v>
+        <f aca="false">Obliczenia!G69</f>
+        <v>247.024096385542</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2753,41 +2759,41 @@
         <v>88</v>
       </c>
       <c r="C14" s="19" t="n">
+        <f aca="false">Obliczenia!D77</f>
+        <v>168.333333333333</v>
+      </c>
+      <c r="D14" s="19" t="n">
+        <f aca="false">Obliczenia!E77</f>
+        <v>168.333333333333</v>
+      </c>
+      <c r="E14" s="19" t="n">
+        <f aca="false">Obliczenia!F77</f>
+        <v>168.333333333333</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <f aca="false">Obliczenia!G77</f>
+        <v>168.333333333333</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" s="19" t="n">
         <f aca="false">Obliczenia!D72</f>
-        <v>1601.80271084337</v>
-      </c>
-      <c r="D14" s="19" t="n">
+        <v>1557.69126506024</v>
+      </c>
+      <c r="D15" s="19" t="n">
         <f aca="false">Obliczenia!E72</f>
-        <v>1601.80271084337</v>
-      </c>
-      <c r="E14" s="19" t="n">
+        <v>1557.69126506024</v>
+      </c>
+      <c r="E15" s="19" t="n">
         <f aca="false">Obliczenia!F72</f>
-        <v>1601.80271084337</v>
-      </c>
-      <c r="F14" s="19" t="n">
+        <v>1557.69126506024</v>
+      </c>
+      <c r="F15" s="19" t="n">
         <f aca="false">Obliczenia!G72</f>
-        <v>1601.80271084337</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="C16" s="19" t="n">
-        <f aca="false">Obliczenia!D54</f>
-        <v>0</v>
-      </c>
-      <c r="D16" s="19" t="n">
-        <f aca="false">Obliczenia!E54</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="19" t="n">
-        <f aca="false">Obliczenia!F54</f>
-        <v>0</v>
-      </c>
-      <c r="F16" s="19" t="n">
-        <f aca="false">Obliczenia!G54</f>
-        <v>0</v>
+        <v>1557.69126506024</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2795,19 +2801,19 @@
         <v>90</v>
       </c>
       <c r="C17" s="19" t="n">
-        <f aca="false">Obliczenia!D55</f>
+        <f aca="false">Obliczenia!D54</f>
         <v>0</v>
       </c>
       <c r="D17" s="19" t="n">
-        <f aca="false">Obliczenia!E55</f>
+        <f aca="false">Obliczenia!E54</f>
         <v>0</v>
       </c>
       <c r="E17" s="19" t="n">
-        <f aca="false">Obliczenia!F55</f>
+        <f aca="false">Obliczenia!F54</f>
         <v>0</v>
       </c>
       <c r="F17" s="19" t="n">
-        <f aca="false">Obliczenia!G55</f>
+        <f aca="false">Obliczenia!G54</f>
         <v>0</v>
       </c>
     </row>
@@ -2816,19 +2822,19 @@
         <v>91</v>
       </c>
       <c r="C18" s="19" t="n">
-        <f aca="false">Obliczenia!D58+Obliczenia!D59+Obliczenia!D60</f>
+        <f aca="false">Obliczenia!D55</f>
         <v>0</v>
       </c>
       <c r="D18" s="19" t="n">
-        <f aca="false">Obliczenia!E58+Obliczenia!E59+Obliczenia!E60</f>
+        <f aca="false">Obliczenia!E55</f>
         <v>0</v>
       </c>
       <c r="E18" s="19" t="n">
-        <f aca="false">Obliczenia!F58+Obliczenia!F59+Obliczenia!F60</f>
+        <f aca="false">Obliczenia!F55</f>
         <v>0</v>
       </c>
       <c r="F18" s="19" t="n">
-        <f aca="false">Obliczenia!G58+Obliczenia!G59+Obliczenia!G60</f>
+        <f aca="false">Obliczenia!G55</f>
         <v>0</v>
       </c>
     </row>
@@ -2837,20 +2843,20 @@
         <v>92</v>
       </c>
       <c r="C19" s="19" t="n">
-        <f aca="false">Obliczenia!D63+Obliczenia!D61+Obliczenia!D62</f>
-        <v>280</v>
+        <f aca="false">Obliczenia!D58+Obliczenia!D59+Obliczenia!D60</f>
+        <v>0</v>
       </c>
       <c r="D19" s="19" t="n">
-        <f aca="false">Obliczenia!E63+Obliczenia!E61+Obliczenia!E62</f>
-        <v>280</v>
+        <f aca="false">Obliczenia!E58+Obliczenia!E59+Obliczenia!E60</f>
+        <v>0</v>
       </c>
       <c r="E19" s="19" t="n">
-        <f aca="false">Obliczenia!F63+Obliczenia!F61+Obliczenia!F62</f>
-        <v>280</v>
+        <f aca="false">Obliczenia!F58+Obliczenia!F59+Obliczenia!F60</f>
+        <v>0</v>
       </c>
       <c r="F19" s="19" t="n">
-        <f aca="false">Obliczenia!G63+Obliczenia!G61+Obliczenia!G62</f>
-        <v>280</v>
+        <f aca="false">Obliczenia!G58+Obliczenia!G59+Obliczenia!G60</f>
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2858,20 +2864,20 @@
         <v>93</v>
       </c>
       <c r="C20" s="19" t="n">
-        <f aca="false">Obliczenia!D57+Obliczenia!D64+Obliczenia!D56</f>
-        <v>1184.5</v>
+        <f aca="false">Obliczenia!D63+Obliczenia!D61+Obliczenia!D62</f>
+        <v>280</v>
       </c>
       <c r="D20" s="19" t="n">
-        <f aca="false">Obliczenia!E57+Obliczenia!E64+Obliczenia!E56</f>
-        <v>1184.5</v>
+        <f aca="false">Obliczenia!E63+Obliczenia!E61+Obliczenia!E62</f>
+        <v>280</v>
       </c>
       <c r="E20" s="19" t="n">
-        <f aca="false">Obliczenia!F57+Obliczenia!F64+Obliczenia!F56</f>
-        <v>1184.5</v>
+        <f aca="false">Obliczenia!F63+Obliczenia!F61+Obliczenia!F62</f>
+        <v>280</v>
       </c>
       <c r="F20" s="19" t="n">
-        <f aca="false">Obliczenia!G57+Obliczenia!G64+Obliczenia!G56</f>
-        <v>1184.5</v>
+        <f aca="false">Obliczenia!G63+Obliczenia!G61+Obliczenia!G62</f>
+        <v>280</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2879,41 +2885,41 @@
         <v>94</v>
       </c>
       <c r="C21" s="19" t="n">
+        <f aca="false">Obliczenia!D57+Obliczenia!D64+Obliczenia!D56</f>
+        <v>1184.5</v>
+      </c>
+      <c r="D21" s="19" t="n">
+        <f aca="false">Obliczenia!E57+Obliczenia!E64+Obliczenia!E56</f>
+        <v>1184.5</v>
+      </c>
+      <c r="E21" s="19" t="n">
+        <f aca="false">Obliczenia!F57+Obliczenia!F64+Obliczenia!F56</f>
+        <v>1184.5</v>
+      </c>
+      <c r="F21" s="19" t="n">
+        <f aca="false">Obliczenia!G57+Obliczenia!G64+Obliczenia!G56</f>
+        <v>1184.5</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" s="19" t="n">
         <f aca="false">Obliczenia!D67+Obliczenia!D68+Obliczenia!D70</f>
         <v>137.302710843374</v>
       </c>
-      <c r="D21" s="19" t="n">
+      <c r="D22" s="19" t="n">
         <f aca="false">Obliczenia!E67+Obliczenia!E68+Obliczenia!E70</f>
         <v>137.302710843374</v>
       </c>
-      <c r="E21" s="19" t="n">
+      <c r="E22" s="19" t="n">
         <f aca="false">Obliczenia!F67+Obliczenia!F68+Obliczenia!F70</f>
         <v>137.302710843374</v>
       </c>
-      <c r="F21" s="19" t="n">
+      <c r="F22" s="19" t="n">
         <f aca="false">Obliczenia!G67+Obliczenia!G68+Obliczenia!G70</f>
         <v>137.302710843374</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="C23" s="21" t="n">
-        <f aca="false">Obliczenia!D51</f>
-        <v>1</v>
-      </c>
-      <c r="D23" s="21" t="n">
-        <f aca="false">Obliczenia!E51</f>
-        <v>1</v>
-      </c>
-      <c r="E23" s="21" t="n">
-        <f aca="false">Obliczenia!F51</f>
-        <v>1</v>
-      </c>
-      <c r="F23" s="21" t="n">
-        <f aca="false">Obliczenia!G51</f>
-        <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2921,65 +2927,73 @@
         <v>96</v>
       </c>
       <c r="C24" s="21" t="n">
+        <f aca="false">Obliczenia!D51</f>
+        <v>1</v>
+      </c>
+      <c r="D24" s="21" t="n">
+        <f aca="false">Obliczenia!E51</f>
+        <v>1</v>
+      </c>
+      <c r="E24" s="21" t="n">
+        <f aca="false">Obliczenia!F51</f>
+        <v>1</v>
+      </c>
+      <c r="F24" s="21" t="n">
+        <f aca="false">Obliczenia!G51</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C25" s="21" t="n">
         <f aca="false">Obliczenia!D52</f>
         <v>1</v>
       </c>
-      <c r="D24" s="21" t="n">
+      <c r="D25" s="21" t="n">
         <f aca="false">Obliczenia!E52</f>
         <v>1</v>
       </c>
-      <c r="E24" s="21" t="n">
+      <c r="E25" s="21" t="n">
         <f aca="false">Obliczenia!F52</f>
         <v>1</v>
       </c>
-      <c r="F24" s="21" t="n">
+      <c r="F25" s="21" t="n">
         <f aca="false">Obliczenia!G52</f>
         <v>1</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="0" t="s">
-        <v>97</v>
-      </c>
-      <c r="C25" s="22" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="C26" s="22" t="n">
         <f aca="false">Obliczenia!D50</f>
         <v>0.7</v>
       </c>
-      <c r="D25" s="22" t="n">
+      <c r="D26" s="22" t="n">
         <f aca="false">Obliczenia!E50</f>
         <v>0.7</v>
       </c>
-      <c r="E25" s="22" t="n">
+      <c r="E26" s="22" t="n">
         <f aca="false">Obliczenia!F50</f>
         <v>0.7</v>
       </c>
-      <c r="F25" s="22" t="n">
+      <c r="F26" s="22" t="n">
         <f aca="false">Obliczenia!G50</f>
         <v>0.7</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C27" s="4" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="C28" s="4" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="0" t="s">
+      <c r="D28" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="C28" s="19" t="n">
-        <f aca="false">Obliczenia!F71-Obliczenia!D71</f>
-        <v>0</v>
-      </c>
-      <c r="D28" s="19" t="n">
-        <f aca="false">Obliczenia!G71-Obliczenia!E71</f>
-        <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2987,11 +3001,11 @@
         <v>102</v>
       </c>
       <c r="C29" s="19" t="n">
-        <f aca="false">Obliczenia!F71-Obliczenia!D71+(c_slupek22-c_slupek)*m_MP*e_mnoznik</f>
+        <f aca="false">Obliczenia!F71-Obliczenia!D71</f>
         <v>0</v>
       </c>
       <c r="D29" s="19" t="n">
-        <f aca="false">Obliczenia!G71-Obliczenia!E71+(c_slupek22-c_slupek)*m_MP*e_mnoznik</f>
+        <f aca="false">Obliczenia!G71-Obliczenia!E71</f>
         <v>0</v>
       </c>
     </row>
@@ -3000,70 +3014,54 @@
         <v>103</v>
       </c>
       <c r="C30" s="19" t="n">
+        <f aca="false">Obliczenia!F71-Obliczenia!D71+(c_slupek22-c_slupek)*m_MP*e_mnoznik</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="19" t="n">
+        <f aca="false">Obliczenia!G71-Obliczenia!E71+(c_slupek22-c_slupek)*m_MP*e_mnoznik</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="C31" s="19" t="n">
         <f aca="false">m_malowanie*e_mnoznik</f>
         <v>0</v>
       </c>
-      <c r="D30" s="19" t="n">
+      <c r="D31" s="19" t="n">
         <f aca="false">m_malowanie*e_mnoznik</f>
         <v>0</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="11" t="str">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="11" t="str">
         <f aca="false">"Analiza liczby osób - wariant: "&amp;in_analiza</f>
         <v>Analiza liczby osób - wariant: 2000 kg</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C33" s="17" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="D33" s="17" t="s">
+      <c r="C34" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="E33" s="17" t="s">
+      <c r="D34" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="F33" s="17" t="s">
+      <c r="E34" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="G33" s="17" t="s">
+      <c r="F34" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="H33" s="17" t="s">
+      <c r="G34" s="17" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="0" t="s">
+      <c r="H34" s="17" t="s">
         <v>111</v>
-      </c>
-      <c r="C34" s="19" t="n">
-        <f aca="false">Obliczenia!I71</f>
-        <v>1018.07954819277</v>
-      </c>
-      <c r="D34" s="19" t="n">
-        <f aca="false">Obliczenia!J71</f>
-        <v>1433.45317771084</v>
-      </c>
-      <c r="E34" s="19" t="n">
-        <f aca="false">Obliczenia!K71</f>
-        <v>1848.82680722892</v>
-      </c>
-      <c r="F34" s="19" t="n">
-        <f aca="false">Obliczenia!L71</f>
-        <v>2264.20043674699</v>
-      </c>
-      <c r="G34" s="19" t="n">
-        <f aca="false">Obliczenia!M71</f>
-        <v>2679.57406626506</v>
-      </c>
-      <c r="H34" s="19" t="n">
-        <f aca="false">Obliczenia!N71</f>
-        <v>3094.94769578313</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3071,85 +3069,85 @@
         <v>112</v>
       </c>
       <c r="C35" s="19" t="n">
-        <f aca="false">Obliczenia!I73</f>
-        <v>0</v>
+        <f aca="false">Obliczenia!I71</f>
+        <v>1018.07954819277</v>
       </c>
       <c r="D35" s="19" t="n">
-        <f aca="false">Obliczenia!J73</f>
-        <v>0</v>
+        <f aca="false">Obliczenia!J71</f>
+        <v>1433.45317771084</v>
       </c>
       <c r="E35" s="19" t="n">
-        <f aca="false">Obliczenia!K73</f>
-        <v>0</v>
+        <f aca="false">Obliczenia!K71</f>
+        <v>1848.82680722892</v>
       </c>
       <c r="F35" s="19" t="n">
-        <f aca="false">Obliczenia!L73</f>
-        <v>0</v>
+        <f aca="false">Obliczenia!L71</f>
+        <v>2264.20043674699</v>
       </c>
       <c r="G35" s="19" t="n">
-        <f aca="false">Obliczenia!M73</f>
-        <v>0</v>
+        <f aca="false">Obliczenia!M71</f>
+        <v>2679.57406626506</v>
       </c>
       <c r="H35" s="19" t="n">
-        <f aca="false">Obliczenia!N73</f>
-        <v>0</v>
+        <f aca="false">Obliczenia!N71</f>
+        <v>3094.94769578313</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="C36" s="23" t="n">
-        <f aca="false">Obliczenia!I51</f>
-        <v>1</v>
-      </c>
-      <c r="D36" s="23" t="n">
-        <f aca="false">Obliczenia!J51</f>
-        <v>1</v>
-      </c>
-      <c r="E36" s="23" t="n">
-        <f aca="false">Obliczenia!K51</f>
-        <v>1</v>
-      </c>
-      <c r="F36" s="23" t="n">
-        <f aca="false">Obliczenia!L51</f>
-        <v>1</v>
-      </c>
-      <c r="G36" s="23" t="n">
-        <f aca="false">Obliczenia!M51</f>
-        <v>1</v>
-      </c>
-      <c r="H36" s="23" t="n">
-        <f aca="false">Obliczenia!N51</f>
-        <v>1</v>
+        <v>113</v>
+      </c>
+      <c r="C36" s="19" t="n">
+        <f aca="false">Obliczenia!I74</f>
+        <v>0</v>
+      </c>
+      <c r="D36" s="19" t="n">
+        <f aca="false">Obliczenia!J74</f>
+        <v>0</v>
+      </c>
+      <c r="E36" s="19" t="n">
+        <f aca="false">Obliczenia!K74</f>
+        <v>0</v>
+      </c>
+      <c r="F36" s="19" t="n">
+        <f aca="false">Obliczenia!L74</f>
+        <v>0</v>
+      </c>
+      <c r="G36" s="19" t="n">
+        <f aca="false">Obliczenia!M74</f>
+        <v>0</v>
+      </c>
+      <c r="H36" s="19" t="n">
+        <f aca="false">Obliczenia!N74</f>
+        <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="0" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="C37" s="23" t="n">
-        <f aca="false">Obliczenia!I48</f>
+        <f aca="false">Obliczenia!I51</f>
         <v>1</v>
       </c>
       <c r="D37" s="23" t="n">
-        <f aca="false">Obliczenia!J48</f>
+        <f aca="false">Obliczenia!J51</f>
         <v>1</v>
       </c>
       <c r="E37" s="23" t="n">
-        <f aca="false">Obliczenia!K48</f>
+        <f aca="false">Obliczenia!K51</f>
         <v>1</v>
       </c>
       <c r="F37" s="23" t="n">
-        <f aca="false">Obliczenia!L48</f>
+        <f aca="false">Obliczenia!L51</f>
         <v>1</v>
       </c>
       <c r="G37" s="23" t="n">
-        <f aca="false">Obliczenia!M48</f>
+        <f aca="false">Obliczenia!M51</f>
         <v>1</v>
       </c>
       <c r="H37" s="23" t="n">
-        <f aca="false">Obliczenia!N48</f>
+        <f aca="false">Obliczenia!N51</f>
         <v>1</v>
       </c>
     </row>
@@ -3157,66 +3155,81 @@
       <c r="B38" s="0" t="s">
         <v>114</v>
       </c>
-      <c r="C38" s="19" t="n">
+      <c r="C38" s="23" t="n">
+        <f aca="false">Obliczenia!I48</f>
+        <v>1</v>
+      </c>
+      <c r="D38" s="23" t="n">
+        <f aca="false">Obliczenia!J48</f>
+        <v>1</v>
+      </c>
+      <c r="E38" s="23" t="n">
+        <f aca="false">Obliczenia!K48</f>
+        <v>1</v>
+      </c>
+      <c r="F38" s="23" t="n">
+        <f aca="false">Obliczenia!L48</f>
+        <v>1</v>
+      </c>
+      <c r="G38" s="23" t="n">
+        <f aca="false">Obliczenia!M48</f>
+        <v>1</v>
+      </c>
+      <c r="H38" s="23" t="n">
+        <f aca="false">Obliczenia!N48</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="C39" s="19" t="n">
         <f aca="false">Obliczenia!I57+Obliczenia!I64</f>
         <v>535.75</v>
       </c>
-      <c r="D38" s="19" t="n">
+      <c r="D39" s="19" t="n">
         <f aca="false">Obliczenia!J57+Obliczenia!J64</f>
         <v>803.625</v>
       </c>
-      <c r="E38" s="19" t="n">
+      <c r="E39" s="19" t="n">
         <f aca="false">Obliczenia!K57+Obliczenia!K64</f>
         <v>1071.5</v>
       </c>
-      <c r="F38" s="19" t="n">
+      <c r="F39" s="19" t="n">
         <f aca="false">Obliczenia!L57+Obliczenia!L64</f>
         <v>1339.375</v>
       </c>
-      <c r="G38" s="19" t="n">
+      <c r="G39" s="19" t="n">
         <f aca="false">Obliczenia!M57+Obliczenia!M64</f>
         <v>1607.25</v>
       </c>
-      <c r="H38" s="19" t="n">
+      <c r="H39" s="19" t="n">
         <f aca="false">Obliczenia!N57+Obliczenia!N64</f>
         <v>1875.125</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="8" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="4" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="C41" s="5"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="0" t="s">
+      <c r="B42" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="C42" s="16" t="str">
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C43" s="16" t="str">
         <f aca="false">in_typ&amp;": "&amp;IF(in_S&gt;0,in_S&amp;" x S (2 MP)  ","")&amp;IF(in_D&gt;0,in_D&amp;" x D (4 MP)  ","")&amp;IF(in_NP&gt;0,in_NP&amp;" x N.P.  ","")&amp;"= "&amp;m_MP&amp;" MP"</f>
         <v>NK38: = 0 MP</v>
-      </c>
-      <c r="D42" s="16"/>
-      <c r="E42" s="16"/>
-      <c r="F42" s="16"/>
-      <c r="G42" s="16"/>
-      <c r="H42" s="16"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="C43" s="16" t="str">
-        <f aca="false">in_agregaty&amp;" szt."</f>
-        <v>0 szt.</v>
       </c>
       <c r="D43" s="16"/>
       <c r="E43" s="16"/>
@@ -3226,11 +3239,11 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="0" t="s">
-        <v>118</v>
+        <v>24</v>
       </c>
       <c r="C44" s="16" t="str">
-        <f aca="false">IF(t_zaglebienia="","standard 170 cm",t_zaglebienia)</f>
-        <v>standard 170 cm</v>
+        <f aca="false">in_agregaty&amp;" szt."</f>
+        <v>0 szt.</v>
       </c>
       <c r="D44" s="16"/>
       <c r="E44" s="16"/>
@@ -3243,8 +3256,8 @@
         <v>119</v>
       </c>
       <c r="C45" s="16" t="str">
-        <f aca="false">IF(t_wymiary="","standard",t_wymiary)</f>
-        <v>standard</v>
+        <f aca="false">IF(t_zaglebienia="","standard 170 cm",t_zaglebienia)</f>
+        <v>standard 170 cm</v>
       </c>
       <c r="D45" s="16"/>
       <c r="E45" s="16"/>
@@ -3257,8 +3270,8 @@
         <v>120</v>
       </c>
       <c r="C46" s="16" t="str">
-        <f aca="false">in_magistrala&amp;" x 6 m  /  "&amp;in_barierki&amp;" szt.  /  "&amp;in_maskownice&amp;" szt."</f>
-        <v>0 x 6 m  /  0 szt.  /  0 szt.</v>
+        <f aca="false">IF(t_wymiary="","standard",t_wymiary)</f>
+        <v>standard</v>
       </c>
       <c r="D46" s="16"/>
       <c r="E46" s="16"/>
@@ -3271,8 +3284,8 @@
         <v>121</v>
       </c>
       <c r="C47" s="16" t="str">
-        <f aca="false">m_utr&amp;" (z magistrali i barierek "&amp;m_utr_auto&amp;", ręcznie "&amp;in_utr_dod&amp;")"</f>
-        <v>0 (z magistrali i barierek 0, ręcznie 0)</v>
+        <f aca="false">in_magistrala&amp;" x 6 m  /  "&amp;in_barierki&amp;" szt.  /  "&amp;in_maskownice&amp;" szt."</f>
+        <v>0 x 6 m  /  0 szt.  /  0 szt.</v>
       </c>
       <c r="D47" s="16"/>
       <c r="E47" s="16"/>
@@ -3282,11 +3295,11 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="0" t="s">
-        <v>10</v>
+        <v>122</v>
       </c>
       <c r="C48" s="16" t="str">
-        <f aca="false">in_lok&amp;IF(e_krk,"","  ("&amp;in_km&amp;" km od Krakowa)")</f>
-        <v>Poza Krakowem  (0 km od Krakowa)</v>
+        <f aca="false">m_utr&amp;" (z magistrali i barierek "&amp;m_utr_auto&amp;", ręcznie "&amp;in_utr_dod&amp;")"</f>
+        <v>0 (z magistrali i barierek 0, ręcznie 0)</v>
       </c>
       <c r="D48" s="16"/>
       <c r="E48" s="16"/>
@@ -3296,11 +3309,11 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="0" t="s">
-        <v>122</v>
+        <v>10</v>
       </c>
       <c r="C49" s="16" t="str">
-        <f aca="false">e_km_pom&amp;" / "&amp;e_km_mon&amp;" km"</f>
-        <v>0 / 50 km</v>
+        <f aca="false">in_lok&amp;IF(e_krk,"","  ("&amp;in_km&amp;" km od Krakowa)")</f>
+        <v>Poza Krakowem  (0 km od Krakowa)</v>
       </c>
       <c r="D49" s="16"/>
       <c r="E49" s="16"/>
@@ -3313,8 +3326,8 @@
         <v>123</v>
       </c>
       <c r="C50" s="16" t="str">
-        <f aca="false">in_tir&amp;" TIR x "&amp;TEXT(in_tir_cena,"#,##0")&amp;" zł, rozładunek sprzętu "&amp;TEXT(in_rozl_cena,"#,##0")&amp;" zł jednorazowo, "&amp;e_rozl_dni&amp;" dni"</f>
-        <v>0 TIR x 0 zł, rozładunek sprzętu 0 zł jednorazowo, 0 dni</v>
+        <f aca="false">e_km_pom&amp;" / "&amp;e_km_mon&amp;" km"</f>
+        <v>0 / 50 km</v>
       </c>
       <c r="D50" s="16"/>
       <c r="E50" s="16"/>
@@ -3327,8 +3340,8 @@
         <v>124</v>
       </c>
       <c r="C51" s="16" t="str">
-        <f aca="false">in_osoby&amp;" osób, średnia stawka "&amp;TEXT(Obliczenia!D41,"#,##0")&amp;" zł/dzień"</f>
-        <v>4 osób, średnia stawka 400 zł/dzień</v>
+        <f aca="false">in_tir&amp;" TIR x "&amp;TEXT(in_tir_cena,"#,##0")&amp;" zł, rozładunek sprzętu "&amp;TEXT(in_rozl_cena,"#,##0")&amp;" zł jednorazowo, "&amp;e_rozl_dni&amp;" dni"</f>
+        <v>0 TIR x 0 zł, rozładunek sprzętu 0 zł jednorazowo, 0 dni</v>
       </c>
       <c r="D51" s="16"/>
       <c r="E51" s="16"/>
@@ -3341,8 +3354,8 @@
         <v>125</v>
       </c>
       <c r="C52" s="16" t="str">
-        <f aca="false">e_dzw_dni&amp;" dni"</f>
-        <v>0 dni</v>
+        <f aca="false">in_osoby&amp;" osób, średnia stawka "&amp;TEXT(Obliczenia!D41,"#,##0")&amp;" zł/dzień"</f>
+        <v>4 osób, średnia stawka 400 zł/dzień</v>
       </c>
       <c r="D52" s="16"/>
       <c r="E52" s="16"/>
@@ -3355,8 +3368,8 @@
         <v>126</v>
       </c>
       <c r="C53" s="16" t="str">
-        <f aca="false">Obliczenia!D51&amp;" dni pracy = "&amp;Obliczenia!D48&amp;IF(e_krk," dni"," tyg.")&amp;", "&amp;TEXT(Obliczenia!D50,"0.0")&amp;" osobodni"</f>
-        <v>1 dni pracy = 1 tyg., 0.7 osobodni</v>
+        <f aca="false">e_dzw_dni&amp;" dni"</f>
+        <v>0 dni</v>
       </c>
       <c r="D53" s="16"/>
       <c r="E53" s="16"/>
@@ -3369,7 +3382,7 @@
         <v>127</v>
       </c>
       <c r="C54" s="16" t="str">
-        <f aca="false">Obliczenia!F51&amp;" dni pracy = "&amp;Obliczenia!F48&amp;IF(e_krk," dni"," tyg.")&amp;", "&amp;TEXT(Obliczenia!F50,"0.0")&amp;" osobodni"</f>
+        <f aca="false">Obliczenia!D51&amp;" dni pracy = "&amp;Obliczenia!D48&amp;IF(e_krk," dni"," tyg.")&amp;", "&amp;TEXT(Obliczenia!D50,"0.0")&amp;" osobodni"</f>
         <v>1 dni pracy = 1 tyg., 0.7 osobodni</v>
       </c>
       <c r="D54" s="16"/>
@@ -3383,8 +3396,8 @@
         <v>128</v>
       </c>
       <c r="C55" s="16" t="str">
-        <f aca="false">TEXT(in_zysk,"0.0%")&amp;" / "&amp;TEXT(in_zysk2,"0.0%")</f>
-        <v>14.0% / 10.0%</v>
+        <f aca="false">Obliczenia!F51&amp;" dni pracy = "&amp;Obliczenia!F48&amp;IF(e_krk," dni"," tyg.")&amp;", "&amp;TEXT(Obliczenia!F50,"0.0")&amp;" osobodni"</f>
+        <v>1 dni pracy = 1 tyg., 0.7 osobodni</v>
       </c>
       <c r="D55" s="16"/>
       <c r="E55" s="16"/>
@@ -3397,8 +3410,8 @@
         <v>129</v>
       </c>
       <c r="C56" s="16" t="str">
-        <f aca="false">TEXT(in_q2500,"0.0%")</f>
-        <v>7.0%</v>
+        <f aca="false">TEXT(in_zysk,"0.0%")&amp;" / "&amp;TEXT(in_zysk2,"0.0%")</f>
+        <v>14.0% / 10.0%</v>
       </c>
       <c r="D56" s="16"/>
       <c r="E56" s="16"/>
@@ -3408,11 +3421,11 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="0" t="s">
-        <v>64</v>
+        <v>130</v>
       </c>
       <c r="C57" s="16" t="str">
-        <f aca="false">in_wzor</f>
-        <v>Stary (poprawiony)</v>
+        <f aca="false">TEXT(in_q2500,"0.0%")</f>
+        <v>7.0%</v>
       </c>
       <c r="D57" s="16"/>
       <c r="E57" s="16"/>
@@ -3422,11 +3435,11 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="0" t="s">
-        <v>130</v>
+        <v>64</v>
       </c>
       <c r="C58" s="16" t="str">
-        <f aca="false">TEXT(in_konsA*m_MP*12,"#,##0")&amp;" / "&amp;TEXT(in_konsB*m_MP*12,"#,##0")&amp;" zł  (przegląd półroczny "&amp;TEXT(in_konsA*m_MP*6,"#,##0")&amp;" / "&amp;TEXT(in_konsB*m_MP*6,"#,##0")&amp;" zł)"</f>
-        <v>0 / 0 zł  (przegląd półroczny 0 / 0 zł)</v>
+        <f aca="false">in_wzor</f>
+        <v>Stary (poprawiony)</v>
       </c>
       <c r="D58" s="16"/>
       <c r="E58" s="16"/>
@@ -3439,8 +3452,8 @@
         <v>131</v>
       </c>
       <c r="C59" s="16" t="str">
-        <f aca="false">in_opis&amp;""</f>
-        <v/>
+        <f aca="false">TEXT(in_konsA*m_MP*12,"#,##0")&amp;" / "&amp;TEXT(in_konsB*m_MP*12,"#,##0")&amp;" zł  (przegląd półroczny "&amp;TEXT(in_konsA*m_MP*6,"#,##0")&amp;" / "&amp;TEXT(in_konsB*m_MP*6,"#,##0")&amp;" zł)"</f>
+        <v>0 / 0 zł  (przegląd półroczny 0 / 0 zł)</v>
       </c>
       <c r="D59" s="16"/>
       <c r="E59" s="16"/>
@@ -3448,36 +3461,39 @@
       <c r="G59" s="16"/>
       <c r="H59" s="16"/>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="11" t="s">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B60" s="0" t="s">
         <v>132</v>
       </c>
-      <c r="C61" s="0" t="str">
+      <c r="C60" s="16" t="str">
+        <f aca="false">in_opis&amp;""</f>
+        <v/>
+      </c>
+      <c r="D60" s="16"/>
+      <c r="E60" s="16"/>
+      <c r="F60" s="16"/>
+      <c r="G60" s="16"/>
+      <c r="H60" s="16"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B62" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="C62" s="0" t="str">
         <f aca="false">IF(COUNTIF(Dane!B66:B71,"ok")=6,"wszystko ok","sprawdź arkusz Dane")</f>
         <v>sprawdź arkusz Dane</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
-      <c r="F63" s="5"/>
-      <c r="G63" s="5"/>
-      <c r="H63" s="5"/>
-    </row>
-    <row r="64" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B64" s="24" t="s">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B64" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="C64" s="24"/>
-      <c r="D64" s="24"/>
-      <c r="E64" s="24"/>
-      <c r="F64" s="24"/>
-      <c r="G64" s="24"/>
-      <c r="H64" s="24"/>
+      <c r="C64" s="5"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="5"/>
+      <c r="H64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="24" t="s">
@@ -3534,9 +3550,19 @@
       <c r="G69" s="24"/>
       <c r="H69" s="24"/>
     </row>
+    <row r="70" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B70" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="C70" s="24"/>
+      <c r="D70" s="24"/>
+      <c r="E70" s="24"/>
+      <c r="F70" s="24"/>
+      <c r="G70" s="24"/>
+      <c r="H70" s="24"/>
+    </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="C42:H42"/>
     <mergeCell ref="C43:H43"/>
     <mergeCell ref="C44:H44"/>
     <mergeCell ref="C45:H45"/>
@@ -3554,21 +3580,22 @@
     <mergeCell ref="C57:H57"/>
     <mergeCell ref="C58:H58"/>
     <mergeCell ref="C59:H59"/>
-    <mergeCell ref="B64:H64"/>
+    <mergeCell ref="C60:H60"/>
     <mergeCell ref="B65:H65"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B67:H67"/>
     <mergeCell ref="B68:H68"/>
     <mergeCell ref="B69:H69"/>
+    <mergeCell ref="B70:H70"/>
   </mergeCells>
-  <conditionalFormatting sqref="C34:H34">
+  <conditionalFormatting sqref="C35:H35">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>C34=MIN($C$34:$H$34)</formula>
+      <formula>C35=MIN($C$35:$H$35)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C61">
+  <conditionalFormatting sqref="C62">
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>C61&lt;&gt;"wszystko ok"</formula>
+      <formula>C62&lt;&gt;"wszystko ok"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3598,7 +3625,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -3607,12 +3634,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -3620,90 +3647,90 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>32500</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>700</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>0.61</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C9" s="14" t="n">
         <v>0.85</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1170</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1560</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1820</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>3110</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3714,34 +3741,34 @@
         <v>2340</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C15" s="25" t="n">
         <v>0.00127</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C16" s="14" t="n">
         <v>0.07</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
@@ -3749,107 +3776,107 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>6500</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1500</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>200</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>500</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>50</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1080</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1175</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1250</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C26" s="26" t="n">
         <f aca="false">0.2*11+0.4*11+2*14+6*11+6*5+6*10</f>
         <v>190.6</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -3857,51 +3884,51 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>600</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>700</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1000</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1800</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
@@ -3909,73 +3936,73 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="0" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>6400</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>13500</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>200</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1700</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>6300</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C38" s="9" t="n">
         <v>0.37</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
@@ -3983,117 +4010,117 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C40" s="9" t="n">
         <v>5.5</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C41" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C42" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C43" s="9" t="n">
         <v>0.5</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C44" s="9" t="n">
         <v>0.5</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C45" s="9" t="n">
         <v>0.5</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>2400</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C47" s="9" t="n">
         <v>5</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C48" s="9" t="n">
         <v>0.6</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C49" s="9" t="n">
         <v>5</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5"/>
@@ -4101,84 +4128,84 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C51" s="9" t="n">
         <v>50</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C52" s="9" t="n">
         <v>20</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C53" s="9" t="n">
         <v>650</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C54" s="9" t="n">
         <v>12</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C55" s="26" t="n">
         <v>9.4</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C56" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C57" s="9" t="n">
         <v>2</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5"/>
@@ -4186,62 +4213,62 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>500</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>400</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C61" s="13" t="n">
         <v>350</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C62" s="13" t="n">
         <v>45</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C63" s="13" t="n">
         <v>130</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C64" s="5"/>
       <c r="D64" s="5"/>
@@ -4249,40 +4276,40 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C65" s="14" t="n">
         <v>0.005</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C66" s="14" t="n">
         <v>0.025</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C67" s="14" t="n">
         <v>0.14</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C69" s="5"/>
       <c r="D69" s="5"/>
@@ -4290,13 +4317,13 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="11" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4400,7 +4427,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C81" s="5"/>
       <c r="D81" s="5"/>
@@ -4409,24 +4436,24 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="11" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C82" s="11" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D82" s="11" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E82" s="11" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F82" s="11" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="0" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C83" s="29" t="n">
         <v>45</v>
@@ -4438,12 +4465,12 @@
         <v>9.6</v>
       </c>
       <c r="F83" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="0" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C84" s="29" t="n">
         <v>8</v>
@@ -4455,12 +4482,12 @@
         <v>4</v>
       </c>
       <c r="F84" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C85" s="29" t="n">
         <v>36</v>
@@ -4472,12 +4499,12 @@
         <v>2</v>
       </c>
       <c r="F85" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C86" s="29" t="n">
         <v>90</v>
@@ -4489,12 +4516,12 @@
         <v>2</v>
       </c>
       <c r="F86" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C87" s="29" t="n">
         <v>207.28</v>
@@ -4506,12 +4533,12 @@
         <v>2</v>
       </c>
       <c r="F87" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="0" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C88" s="29" t="n">
         <v>40.14</v>
@@ -4523,12 +4550,12 @@
         <v>2</v>
       </c>
       <c r="F88" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="0" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C89" s="29" t="n">
         <v>3.3</v>
@@ -4540,12 +4567,12 @@
         <v>2</v>
       </c>
       <c r="F89" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="0" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C90" s="29" t="n">
         <v>10.8</v>
@@ -4557,12 +4584,12 @@
         <v>2</v>
       </c>
       <c r="F90" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="0" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C91" s="29" t="n">
         <v>10.95</v>
@@ -4574,12 +4601,12 @@
         <v>2</v>
       </c>
       <c r="F91" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="0" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C92" s="29" t="n">
         <v>3.81</v>
@@ -4591,12 +4618,12 @@
         <v>2</v>
       </c>
       <c r="F92" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="0" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C93" s="29" t="n">
         <v>2.84</v>
@@ -4608,12 +4635,12 @@
         <v>4</v>
       </c>
       <c r="F93" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="0" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C94" s="29" t="n">
         <v>4.4</v>
@@ -4625,12 +4652,12 @@
         <v>4</v>
       </c>
       <c r="F94" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="0" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C95" s="29" t="n">
         <f aca="false">2*25.71+2*22.85</f>
@@ -4643,12 +4670,12 @@
         <v>1</v>
       </c>
       <c r="F95" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="0" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C96" s="29" t="n">
         <v>345</v>
@@ -4660,12 +4687,12 @@
         <v>0</v>
       </c>
       <c r="F96" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="0" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C97" s="29" t="n">
         <v>546</v>
@@ -4677,12 +4704,12 @@
         <v>1</v>
       </c>
       <c r="F97" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="0" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C98" s="29" t="n">
         <v>2.98</v>
@@ -4694,12 +4721,12 @@
         <v>208</v>
       </c>
       <c r="F98" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="0" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C99" s="29" t="n">
         <f aca="false">3.09+4.99</f>
@@ -4712,12 +4739,12 @@
         <v>20</v>
       </c>
       <c r="F99" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B100" s="0" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C100" s="29" t="n">
         <v>5.4</v>
@@ -4729,12 +4756,12 @@
         <v>1</v>
       </c>
       <c r="F100" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B101" s="0" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C101" s="29" t="n">
         <v>300</v>
@@ -4746,12 +4773,12 @@
         <v>1</v>
       </c>
       <c r="F101" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B102" s="0" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C102" s="29" t="n">
         <v>40</v>
@@ -4763,12 +4790,12 @@
         <v>1</v>
       </c>
       <c r="F102" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B103" s="0" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C103" s="29" t="n">
         <v>172</v>
@@ -4780,12 +4807,12 @@
         <v>0</v>
       </c>
       <c r="F103" s="30" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B104" s="0" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C104" s="29" t="n">
         <v>207</v>
@@ -4797,12 +4824,12 @@
         <v>1</v>
       </c>
       <c r="F104" s="30" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="0" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C105" s="29" t="n">
         <f aca="false">120+55+65</f>
@@ -4815,12 +4842,12 @@
         <v>1</v>
       </c>
       <c r="F105" s="30" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B106" s="0" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C106" s="29" t="n">
         <f aca="false">50+40</f>
@@ -4833,12 +4860,12 @@
         <v>1</v>
       </c>
       <c r="F106" s="30" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B107" s="0" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C107" s="29" t="n">
         <f aca="false">14+9+25+5+9+30</f>
@@ -4851,12 +4878,12 @@
         <v>0</v>
       </c>
       <c r="F107" s="30" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B108" s="0" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C108" s="29" t="n">
         <f aca="false">14+18+25+7+18+30</f>
@@ -4869,12 +4896,12 @@
         <v>1</v>
       </c>
       <c r="F108" s="30" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="0" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C109" s="29" t="n">
         <f aca="false">70+14+34+32+20</f>
@@ -4887,7 +4914,7 @@
         <v>1</v>
       </c>
       <c r="F109" s="30" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -4906,7 +4933,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:N78"/>
+  <dimension ref="B2:N79"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -4918,7 +4945,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -4935,13 +4962,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="0" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C5" s="31" t="n">
         <f aca="false">c_cena_D+IF(in_typ="NK37",c_doplata_NK37,0)</f>
@@ -4950,7 +4977,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="0" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C6" s="31" t="n">
         <f aca="false">c_wsp_S*m_cena_D</f>
@@ -4959,7 +4986,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="0" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C7" s="31" t="n">
         <f aca="false">c_wsp_NP*m_cena_D</f>
@@ -4968,7 +4995,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="0" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C8" s="32" t="n">
         <f aca="false">in_D+in_NP</f>
@@ -4977,7 +5004,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="0" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C9" s="32" t="n">
         <f aca="false">in_S+in_D+in_NP</f>
@@ -4986,7 +5013,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="0" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C10" s="32" t="n">
         <f aca="false">2*in_S+2*in_NP+4*in_D</f>
@@ -4995,7 +5022,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="0" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C11" s="31" t="n">
         <f aca="false">m_cena_S*in_S+c_szer_260*in_szer1_S+c_szer_270*in_szer2_S+SUMPRODUCT(in_gl_S,t_gl_doplata)+c_dl_500*in_dl500_S+CEILING(m_cena_S*c_dl_wsp*10,100)*in_dl540_S+CEILING(m_cena_S*c_dl_wsp*20,100)*in_dl550_S</f>
@@ -5004,7 +5031,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="0" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C12" s="31" t="n">
         <f aca="false">m_cena_D*in_D+c_szer_520*in_szer1_D+c_szer_540*in_szer2_D+SUMPRODUCT(in_gl_D,t_gl_doplata)+c_dl_500*in_dl500_D+m_cena_D*c_dl_wsp*10*in_dl540_D+m_cena_D*c_dl_wsp*20*in_dl550_D</f>
@@ -5013,7 +5040,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="0" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C13" s="31" t="n">
         <f aca="false">m_cena_NP*in_NP</f>
@@ -5022,7 +5049,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="0" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C14" s="32" t="n">
         <f aca="false">SUMPRODUCT((t_gl_silownik=2000)*(in_gl_S+in_gl_D))</f>
@@ -5031,7 +5058,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="0" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C15" s="32" t="n">
         <f aca="false">SUMPRODUCT((t_gl_silownik=2250)*(in_gl_S+in_gl_D))</f>
@@ -5040,7 +5067,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="0" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C16" s="32" t="n">
         <f aca="false">m_platformy-m_sil_2000-m_sil_2250</f>
@@ -5049,7 +5076,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C17" s="31" t="n">
         <f aca="false">in_agregaty*(c_agregat+c_hydr_drobne+c_olej+c_transp_agregatu)+m_platformy*c_transp_silownikow+2*(c_sil_1700*m_sil_std+c_sil_2000*m_sil_2000+c_sil_2250*m_sil_2250)+in_magistrala*c_magistrala+SUMPRODUCT((t_sk_grupa="Hydraulika")*t_sk_cena*(t_sk_S*in_S+t_sk_D*m_DN))</f>
@@ -5058,7 +5085,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="0" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C18" s="31" t="n">
         <f aca="false">in_barierki*c_barierka+in_maskownice*c_maskownica</f>
@@ -5067,7 +5094,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="0" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C19" s="31" t="n">
         <f aca="false">in_agregaty*c_skrzynka_zasil+SUMPRODUCT((t_sk_grupa="Elektryka")*t_sk_cena*(t_sk_S*in_S+t_sk_D*m_DN))</f>
@@ -5076,7 +5103,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="0" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C20" s="31" t="n">
         <f aca="false">in_agregaty*c_admin+SUMPRODUCT((t_sk_grupa="Mechanika")*t_sk_cena*(t_sk_S*in_S+t_sk_D*m_DN))</f>
@@ -5085,7 +5112,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C21" s="33" t="n">
         <f aca="false">m_plat_S+m_plat_D+m_plat_NP+m_hydraulika+m_barierki+m_elektryka+m_mechanika</f>
@@ -5094,7 +5121,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C22" s="33" t="n">
         <f aca="false">m_suma_2000*(1+in_q2500)</f>
@@ -5103,7 +5130,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="0" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C23" s="31" t="n">
         <f aca="false">c_mal_S*in_S+c_mal_D*m_DN+c_mal_bar*in_barierki</f>
@@ -5112,7 +5139,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="0" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C24" s="34" t="n">
         <f aca="false">ROUNDUP(in_magistrala*c_osd_magistrala+(in_barierki+in_maskownice)*c_osd_barierka,0)</f>
@@ -5121,7 +5148,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="0" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C25" s="34" t="n">
         <f aca="false">m_utr_auto+in_utr_dod</f>
@@ -5130,13 +5157,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="0" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C28" s="35" t="b">
         <f aca="false">in_lok="Kraków"</f>
@@ -5145,7 +5172,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="0" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C29" s="34" t="n">
         <f aca="false">IF(ISBLANK(in_km_pom),IF(e_krk,c_km_krakow,in_km),in_km_pom)</f>
@@ -5154,7 +5181,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="0" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C30" s="34" t="n">
         <f aca="false">IF(ISBLANK(in_km_mon),IF(e_krk,c_km_krakow,in_km+c_km_dodatek),in_km_mon)</f>
@@ -5163,7 +5190,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="0" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C31" s="34" t="n">
         <f aca="false">IF(ISBLANK(in_rozl_dni),c_rozl_TIR*in_tir,in_rozl_dni)</f>
@@ -5172,7 +5199,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="0" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C32" s="34" t="n">
         <f aca="false">(c_pomiary_osoby+c_odbiory_osoby)*IF(in_wzor="Uproszczony",2*e_km_pom/c_km_dzien*1,(1+0.1*MAX(0,800-e_km_pom)/100)*e_km_pom*1/500)</f>
@@ -5181,7 +5208,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="0" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C33" s="32" t="n">
         <f aca="false">ROUNDUP(m_DN/c_dzwig_D+in_S*c_dzwig_wspS/c_dzwig_D,0)</f>
@@ -5190,7 +5217,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C34" s="36" t="n">
         <f aca="false">(1+c_podatek*(c_gdw+in_zysk))/(1-(c_kob+c_gdw+in_zysk))</f>
@@ -5199,7 +5226,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
@@ -5208,7 +5235,7 @@
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
       <c r="I36" s="4" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="J36" s="5"/>
       <c r="K36" s="5"/>
@@ -5218,7 +5245,7 @@
     </row>
     <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D37" s="37" t="s">
         <v>76</v>
@@ -5233,27 +5260,27 @@
         <v>82</v>
       </c>
       <c r="I37" s="37" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J37" s="37" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K37" s="37" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L37" s="37" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="M37" s="37" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N37" s="37" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="0" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D38" s="32" t="n">
         <v>0</v>
@@ -5294,7 +5321,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="0" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D39" s="32" t="n">
         <v>0</v>
@@ -5335,7 +5362,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D40" s="32" t="n">
         <f aca="false">in_osoby</f>
@@ -5374,7 +5401,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="0" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D41" s="31" t="n">
         <f aca="false">(c_stawka_1+IF(D40&gt;=2,c_stawka_2,0)+MAX(0,D40-2)*c_stawka_n)/D40</f>
@@ -5419,7 +5446,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="0" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D42" s="34" t="n">
         <f aca="false">c_osd_S*in_S+c_osd_D*in_D+c_osd_NP*in_NP+m_utr+D39*c_slupek_rbd*m_MP</f>
@@ -5464,7 +5491,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="0" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D43" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*1,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*1/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*1,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*1/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5509,7 +5536,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="0" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D44" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D43,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D43/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D43,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D43/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5554,7 +5581,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="0" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D45" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D44,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D44/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D44,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D44/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5599,7 +5626,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="0" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D46" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D45,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D45/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D45,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D45/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5644,7 +5671,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="0" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D47" s="32" t="n">
         <f aca="false">IF(e_krk,CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D46,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D46/500))))/D40,1),CEILING(CEILING((D42+(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D46,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D46/500))))/D40,1)/c_dni_tydzien,1))</f>
@@ -5689,7 +5716,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D48" s="38" t="n">
         <f aca="false">IF(ISBLANK(in_wyjazdy),D47,in_wyjazdy)</f>
@@ -5734,7 +5761,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="0" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D49" s="34" t="n">
         <f aca="false">(e_podr_pom+D40*(e_rozl_dni+IF(in_wzor="Uproszczony",2*e_km_mon/c_km_dzien*D48,(1+0.1*MAX(0,800-e_km_mon)/100)*e_km_mon*D48/500)))</f>
@@ -5779,7 +5806,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D50" s="34" t="n">
         <f aca="false">D42+D49</f>
@@ -5824,7 +5851,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D51" s="38" t="n">
         <f aca="false">CEILING(D50/D40,1)</f>
@@ -5869,7 +5896,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D52" s="38" t="n">
         <f aca="false">IF(e_krk,CEILING(D51/c_dni_tydzien,1),D48)</f>
@@ -5914,7 +5941,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="0" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D53" s="34" t="n">
         <f aca="false">2*(e_km_mon*D48+2*e_km_pom)</f>
@@ -5959,7 +5986,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D54" s="31" t="n">
         <f aca="false">IF(D38=1,m_suma_2500,m_suma_2000)</f>
@@ -6004,7 +6031,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D55" s="31" t="n">
         <f aca="false">D39*c_slupek*m_MP</f>
@@ -6049,7 +6076,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="0" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D56" s="31" t="n">
         <f aca="false">D53/100*ROUNDUP(c_spalanie*c_paliwo,0)</f>
@@ -6094,7 +6121,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="0" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D57" s="31" t="n">
         <f aca="false">IF(e_krk,0,c_hotel*(D51+1)*D40)</f>
@@ -6139,7 +6166,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="0" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D58" s="31" t="n">
         <f aca="false">in_tir_cena*in_tir</f>
@@ -6184,7 +6211,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="0" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D59" s="31" t="n">
         <f aca="false">IF(ISBLANK(in_dzwig_koszt),c_dzwig*e_dzw_dni,in_dzwig_koszt)</f>
@@ -6229,7 +6256,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="0" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D60" s="31" t="n">
         <f aca="false">in_rozl_cena</f>
@@ -6274,7 +6301,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="0" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D61" s="31" t="n">
         <f aca="false">D41*e_rozl_dni*D40</f>
@@ -6319,7 +6346,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="0" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D62" s="31" t="n">
         <f aca="false">D41*(D49-D40*e_rozl_dni)</f>
@@ -6364,7 +6391,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="0" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D63" s="31" t="n">
         <f aca="false">IF(D48&gt;0,D41*D42,0)</f>
@@ -6409,7 +6436,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="0" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D64" s="31" t="n">
         <f aca="false">IF(e_krk,0,c_dieta*D50)</f>
@@ -6454,7 +6481,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D65" s="33" t="n">
         <f aca="false">SUM(D54:D64)</f>
@@ -6499,7 +6526,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="0" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D66" s="31" t="n">
         <f aca="false">D65/(1-(c_kob+c_gdw+in_zysk))</f>
@@ -6544,7 +6571,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="0" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D67" s="31" t="n">
         <f aca="false">D66*c_kob</f>
@@ -6589,7 +6616,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="0" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D68" s="31" t="n">
         <f aca="false">D66*c_gdw</f>
@@ -6634,7 +6661,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="0" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D69" s="31" t="n">
         <f aca="false">D66*in_zysk</f>
@@ -6679,7 +6706,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="0" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D70" s="31" t="n">
         <f aca="false">c_podatek*(D61+D62+D63+D64+D68+D69)</f>
@@ -6724,7 +6751,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D71" s="33" t="n">
         <f aca="false">D66+D70</f>
@@ -6769,316 +6796,361 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="0" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D72" s="31" t="n">
-        <f aca="false">D71-D69</f>
-        <v>1601.80271084337</v>
+        <f aca="false">D71-D69-D68</f>
+        <v>1557.69126506024</v>
       </c>
       <c r="E72" s="31" t="n">
-        <f aca="false">E71-E69</f>
-        <v>1601.80271084337</v>
+        <f aca="false">E71-E69-E68</f>
+        <v>1557.69126506024</v>
       </c>
       <c r="F72" s="31" t="n">
-        <f aca="false">F71-F69</f>
-        <v>1601.80271084337</v>
+        <f aca="false">F71-F69-F68</f>
+        <v>1557.69126506024</v>
       </c>
       <c r="G72" s="31" t="n">
-        <f aca="false">G71-G69</f>
-        <v>1601.80271084337</v>
+        <f aca="false">G71-G69-G68</f>
+        <v>1557.69126506024</v>
       </c>
       <c r="I72" s="31" t="n">
-        <f aca="false">I71-I69</f>
-        <v>882.085572289157</v>
+        <f aca="false">I71-I69-I68</f>
+        <v>857.80093373494</v>
       </c>
       <c r="J72" s="31" t="n">
-        <f aca="false">J71-J69</f>
-        <v>1241.94414156627</v>
+        <f aca="false">J71-J69-J68</f>
+        <v>1207.74609939759</v>
       </c>
       <c r="K72" s="31" t="n">
-        <f aca="false">K71-K69</f>
-        <v>1601.80271084337</v>
+        <f aca="false">K71-K69-K68</f>
+        <v>1557.69126506024</v>
       </c>
       <c r="L72" s="31" t="n">
-        <f aca="false">L71-L69</f>
-        <v>1961.66128012048</v>
+        <f aca="false">L71-L69-L68</f>
+        <v>1907.63643072289</v>
       </c>
       <c r="M72" s="31" t="n">
-        <f aca="false">M71-M69</f>
-        <v>2321.51984939759</v>
+        <f aca="false">M71-M69-M68</f>
+        <v>2257.58159638554</v>
       </c>
       <c r="N72" s="31" t="n">
-        <f aca="false">N71-N69</f>
-        <v>2681.3784186747</v>
+        <f aca="false">N71-N69-N68</f>
+        <v>2607.52676204819</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B73" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="D73" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,D71/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="E73" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,E71/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F73" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,F71/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="G73" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,G71/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="I73" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,I71/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="J73" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,J71/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="K73" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,K71/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="L73" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,L71/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="M73" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,M71/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N73" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,N71/m_MP,0)</f>
-        <v>0</v>
+      <c r="B73" s="11" t="s">
+        <v>357</v>
+      </c>
+      <c r="D73" s="33" t="n">
+        <f aca="false">D71-D72</f>
+        <v>291.135542168675</v>
+      </c>
+      <c r="E73" s="33" t="n">
+        <f aca="false">E71-E72</f>
+        <v>291.135542168675</v>
+      </c>
+      <c r="F73" s="33" t="n">
+        <f aca="false">F71-F72</f>
+        <v>291.135542168675</v>
+      </c>
+      <c r="G73" s="33" t="n">
+        <f aca="false">G71-G72</f>
+        <v>291.135542168675</v>
+      </c>
+      <c r="I73" s="33" t="n">
+        <f aca="false">I71-I72</f>
+        <v>160.278614457831</v>
+      </c>
+      <c r="J73" s="33" t="n">
+        <f aca="false">J71-J72</f>
+        <v>225.707078313253</v>
+      </c>
+      <c r="K73" s="33" t="n">
+        <f aca="false">K71-K72</f>
+        <v>291.135542168675</v>
+      </c>
+      <c r="L73" s="33" t="n">
+        <f aca="false">L71-L72</f>
+        <v>356.564006024096</v>
+      </c>
+      <c r="M73" s="33" t="n">
+        <f aca="false">M71-M72</f>
+        <v>421.992469879518</v>
+      </c>
+      <c r="N73" s="33" t="n">
+        <f aca="false">N71-N72</f>
+        <v>487.42093373494</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="0" t="s">
-        <v>356</v>
-      </c>
-      <c r="D74" s="39" t="n">
-        <f aca="false">D73/in_eur</f>
-        <v>0</v>
-      </c>
-      <c r="E74" s="39" t="n">
-        <f aca="false">E73/in_eur</f>
-        <v>0</v>
-      </c>
-      <c r="F74" s="39" t="n">
-        <f aca="false">F73/in_eur</f>
-        <v>0</v>
-      </c>
-      <c r="G74" s="39" t="n">
-        <f aca="false">G73/in_eur</f>
-        <v>0</v>
-      </c>
-      <c r="I74" s="39" t="n">
-        <f aca="false">I73/in_eur</f>
-        <v>0</v>
-      </c>
-      <c r="J74" s="39" t="n">
-        <f aca="false">J73/in_eur</f>
-        <v>0</v>
-      </c>
-      <c r="K74" s="39" t="n">
-        <f aca="false">K73/in_eur</f>
-        <v>0</v>
-      </c>
-      <c r="L74" s="39" t="n">
-        <f aca="false">L73/in_eur</f>
-        <v>0</v>
-      </c>
-      <c r="M74" s="39" t="n">
-        <f aca="false">M73/in_eur</f>
-        <v>0</v>
-      </c>
-      <c r="N74" s="39" t="n">
-        <f aca="false">N73/in_eur</f>
+        <v>113</v>
+      </c>
+      <c r="D74" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,D71/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E74" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,E71/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F74" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,F71/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G74" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,G71/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I74" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,I71/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J74" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,J71/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K74" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,K71/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L74" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,L71/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M74" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,M71/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N74" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,N71/m_MP,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="0" t="s">
-        <v>357</v>
-      </c>
-      <c r="D75" s="31" t="n">
+        <v>358</v>
+      </c>
+      <c r="D75" s="39" t="n">
+        <f aca="false">D74/in_eur</f>
+        <v>0</v>
+      </c>
+      <c r="E75" s="39" t="n">
+        <f aca="false">E74/in_eur</f>
+        <v>0</v>
+      </c>
+      <c r="F75" s="39" t="n">
+        <f aca="false">F74/in_eur</f>
+        <v>0</v>
+      </c>
+      <c r="G75" s="39" t="n">
+        <f aca="false">G74/in_eur</f>
+        <v>0</v>
+      </c>
+      <c r="I75" s="39" t="n">
+        <f aca="false">I74/in_eur</f>
+        <v>0</v>
+      </c>
+      <c r="J75" s="39" t="n">
+        <f aca="false">J74/in_eur</f>
+        <v>0</v>
+      </c>
+      <c r="K75" s="39" t="n">
+        <f aca="false">K74/in_eur</f>
+        <v>0</v>
+      </c>
+      <c r="L75" s="39" t="n">
+        <f aca="false">L74/in_eur</f>
+        <v>0</v>
+      </c>
+      <c r="M75" s="39" t="n">
+        <f aca="false">M74/in_eur</f>
+        <v>0</v>
+      </c>
+      <c r="N75" s="39" t="n">
+        <f aca="false">N74/in_eur</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B76" s="0" t="s">
+        <v>359</v>
+      </c>
+      <c r="D76" s="31" t="n">
         <f aca="false">D65/(1-(c_kob+c_gdw+in_zysk2))</f>
         <v>1683.33333333333</v>
       </c>
-      <c r="E75" s="31" t="n">
+      <c r="E76" s="31" t="n">
         <f aca="false">E65/(1-(c_kob+c_gdw+in_zysk2))</f>
         <v>1683.33333333333</v>
       </c>
-      <c r="F75" s="31" t="n">
+      <c r="F76" s="31" t="n">
         <f aca="false">F65/(1-(c_kob+c_gdw+in_zysk2))</f>
         <v>1683.33333333333</v>
       </c>
-      <c r="G75" s="31" t="n">
+      <c r="G76" s="31" t="n">
         <f aca="false">G65/(1-(c_kob+c_gdw+in_zysk2))</f>
         <v>1683.33333333333</v>
       </c>
-      <c r="I75" s="31" t="n">
+      <c r="I76" s="31" t="n">
         <f aca="false">I65/(1-(c_kob+c_gdw+in_zysk2))</f>
         <v>926.724137931035</v>
       </c>
-      <c r="J75" s="31" t="n">
+      <c r="J76" s="31" t="n">
         <f aca="false">J65/(1-(c_kob+c_gdw+in_zysk2))</f>
         <v>1305.02873563218</v>
       </c>
-      <c r="K75" s="31" t="n">
+      <c r="K76" s="31" t="n">
         <f aca="false">K65/(1-(c_kob+c_gdw+in_zysk2))</f>
         <v>1683.33333333333</v>
       </c>
-      <c r="L75" s="31" t="n">
+      <c r="L76" s="31" t="n">
         <f aca="false">L65/(1-(c_kob+c_gdw+in_zysk2))</f>
         <v>2061.63793103448</v>
       </c>
-      <c r="M75" s="31" t="n">
+      <c r="M76" s="31" t="n">
         <f aca="false">M65/(1-(c_kob+c_gdw+in_zysk2))</f>
         <v>2439.94252873563</v>
       </c>
-      <c r="N75" s="31" t="n">
+      <c r="N76" s="31" t="n">
         <f aca="false">N65/(1-(c_kob+c_gdw+in_zysk2))</f>
         <v>2818.24712643678</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B76" s="0" t="s">
-        <v>358</v>
-      </c>
-      <c r="D76" s="31" t="n">
-        <f aca="false">D75*in_zysk2</f>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B77" s="0" t="s">
+        <v>360</v>
+      </c>
+      <c r="D77" s="31" t="n">
+        <f aca="false">D76*in_zysk2</f>
         <v>168.333333333333</v>
       </c>
-      <c r="E76" s="31" t="n">
-        <f aca="false">E75*in_zysk2</f>
+      <c r="E77" s="31" t="n">
+        <f aca="false">E76*in_zysk2</f>
         <v>168.333333333333</v>
       </c>
-      <c r="F76" s="31" t="n">
-        <f aca="false">F75*in_zysk2</f>
+      <c r="F77" s="31" t="n">
+        <f aca="false">F76*in_zysk2</f>
         <v>168.333333333333</v>
       </c>
-      <c r="G76" s="31" t="n">
-        <f aca="false">G75*in_zysk2</f>
+      <c r="G77" s="31" t="n">
+        <f aca="false">G76*in_zysk2</f>
         <v>168.333333333333</v>
       </c>
-      <c r="I76" s="31" t="n">
-        <f aca="false">I75*in_zysk2</f>
+      <c r="I77" s="31" t="n">
+        <f aca="false">I76*in_zysk2</f>
         <v>92.6724137931035</v>
       </c>
-      <c r="J76" s="31" t="n">
-        <f aca="false">J75*in_zysk2</f>
+      <c r="J77" s="31" t="n">
+        <f aca="false">J76*in_zysk2</f>
         <v>130.502873563218</v>
       </c>
-      <c r="K76" s="31" t="n">
-        <f aca="false">K75*in_zysk2</f>
+      <c r="K77" s="31" t="n">
+        <f aca="false">K76*in_zysk2</f>
         <v>168.333333333333</v>
       </c>
-      <c r="L76" s="31" t="n">
-        <f aca="false">L75*in_zysk2</f>
+      <c r="L77" s="31" t="n">
+        <f aca="false">L76*in_zysk2</f>
         <v>206.163793103448</v>
       </c>
-      <c r="M76" s="31" t="n">
-        <f aca="false">M75*in_zysk2</f>
+      <c r="M77" s="31" t="n">
+        <f aca="false">M76*in_zysk2</f>
         <v>243.994252873563</v>
       </c>
-      <c r="N76" s="31" t="n">
-        <f aca="false">N75*in_zysk2</f>
+      <c r="N77" s="31" t="n">
+        <f aca="false">N76*in_zysk2</f>
         <v>281.824712643678</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B77" s="11" t="s">
-        <v>359</v>
-      </c>
-      <c r="D77" s="33" t="n">
-        <f aca="false">D75+c_podatek*(D61+D62+D63+D64+D75*(c_gdw+in_zysk2))</f>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B78" s="11" t="s">
+        <v>361</v>
+      </c>
+      <c r="D78" s="33" t="n">
+        <f aca="false">D76+c_podatek*(D61+D62+D63+D64+D76*(c_gdw+in_zysk2))</f>
         <v>1756.40166666667</v>
       </c>
-      <c r="E77" s="33" t="n">
-        <f aca="false">E75+c_podatek*(E61+E62+E63+E64+E75*(c_gdw+in_zysk2))</f>
+      <c r="E78" s="33" t="n">
+        <f aca="false">E76+c_podatek*(E61+E62+E63+E64+E76*(c_gdw+in_zysk2))</f>
         <v>1756.40166666667</v>
       </c>
-      <c r="F77" s="33" t="n">
-        <f aca="false">F75+c_podatek*(F61+F62+F63+F64+F75*(c_gdw+in_zysk2))</f>
+      <c r="F78" s="33" t="n">
+        <f aca="false">F76+c_podatek*(F61+F62+F63+F64+F76*(c_gdw+in_zysk2))</f>
         <v>1756.40166666667</v>
       </c>
-      <c r="G77" s="33" t="n">
-        <f aca="false">G75+c_podatek*(G61+G62+G63+G64+G75*(c_gdw+in_zysk2))</f>
+      <c r="G78" s="33" t="n">
+        <f aca="false">G76+c_podatek*(G61+G62+G63+G64+G76*(c_gdw+in_zysk2))</f>
         <v>1756.40166666667</v>
       </c>
-      <c r="I77" s="33" t="n">
-        <f aca="false">I75+c_podatek*(I61+I62+I63+I64+I75*(c_gdw+in_zysk2))</f>
+      <c r="I78" s="33" t="n">
+        <f aca="false">I76+c_podatek*(I61+I62+I63+I64+I76*(c_gdw+in_zysk2))</f>
         <v>967.196810344828</v>
       </c>
-      <c r="J77" s="33" t="n">
-        <f aca="false">J75+c_podatek*(J61+J62+J63+J64+J75*(c_gdw+in_zysk2))</f>
+      <c r="J78" s="33" t="n">
+        <f aca="false">J76+c_podatek*(J61+J62+J63+J64+J76*(c_gdw+in_zysk2))</f>
         <v>1361.79923850575</v>
       </c>
-      <c r="K77" s="33" t="n">
-        <f aca="false">K75+c_podatek*(K61+K62+K63+K64+K75*(c_gdw+in_zysk2))</f>
+      <c r="K78" s="33" t="n">
+        <f aca="false">K76+c_podatek*(K61+K62+K63+K64+K76*(c_gdw+in_zysk2))</f>
         <v>1756.40166666667</v>
       </c>
-      <c r="L77" s="33" t="n">
-        <f aca="false">L75+c_podatek*(L61+L62+L63+L64+L75*(c_gdw+in_zysk2))</f>
+      <c r="L78" s="33" t="n">
+        <f aca="false">L76+c_podatek*(L61+L62+L63+L64+L76*(c_gdw+in_zysk2))</f>
         <v>2151.00409482759</v>
       </c>
-      <c r="M77" s="33" t="n">
-        <f aca="false">M75+c_podatek*(M61+M62+M63+M64+M75*(c_gdw+in_zysk2))</f>
+      <c r="M78" s="33" t="n">
+        <f aca="false">M76+c_podatek*(M61+M62+M63+M64+M76*(c_gdw+in_zysk2))</f>
         <v>2545.60652298851</v>
       </c>
-      <c r="N77" s="33" t="n">
-        <f aca="false">N75+c_podatek*(N61+N62+N63+N64+N75*(c_gdw+in_zysk2))</f>
+      <c r="N78" s="33" t="n">
+        <f aca="false">N76+c_podatek*(N61+N62+N63+N64+N76*(c_gdw+in_zysk2))</f>
         <v>2940.20895114943</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B78" s="0" t="s">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B79" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="D78" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,D77/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="E78" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,E77/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F78" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,F77/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="G78" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,G77/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="I78" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,I77/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="J78" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,J77/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="K78" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,K77/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="L78" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,L77/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="M78" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,M77/m_MP,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N78" s="31" t="n">
-        <f aca="false">IF(m_MP&gt;0,N77/m_MP,0)</f>
+      <c r="D79" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,D78/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E79" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,E78/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F79" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,F78/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G79" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,G78/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I79" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,I78/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J79" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,J78/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K79" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,K78/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L79" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,L78/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M79" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,M78/m_MP,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N79" s="31" t="n">
+        <f aca="false">IF(m_MP&gt;0,N78/m_MP,0)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>